<commit_message>
Structure prototypes for animations
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -18,7 +18,8 @@
     <sheet state="visible" name="TYPES" sheetId="13" r:id="rId17"/>
     <sheet state="visible" name="EVENTS" sheetId="14" r:id="rId18"/>
     <sheet state="visible" name="DETAILS" sheetId="15" r:id="rId19"/>
-    <sheet state="visible" name="_TODO" sheetId="16" r:id="rId20"/>
+    <sheet state="visible" name="ANIMATIONS" sheetId="16" r:id="rId20"/>
+    <sheet state="visible" name="_TODO" sheetId="17" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="Interval_autoInsertMemento">FN!$A$10:$E$11</definedName>
@@ -122,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3915" uniqueCount="1395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3919" uniqueCount="1397">
   <si>
     <t>NewItem</t>
   </si>
@@ -4205,6 +4206,12 @@
   </si>
   <si>
     <t>DETAIL_LAST</t>
+  </si>
+  <si>
+    <t>ANIMATION_NONE</t>
+  </si>
+  <si>
+    <t>ANIMATION_LAST</t>
   </si>
   <si>
     <t>TASK</t>
@@ -4678,7 +4685,7 @@
       <border/>
     </dxf>
   </dxfs>
-  <tableStyles count="32">
+  <tableStyles count="33">
     <tableStyle count="4" pivot="0" name="FN-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
@@ -4860,6 +4867,12 @@
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
     <tableStyle count="4" pivot="0" name="DETAILS-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="ANIMATIONS-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -5473,6 +5486,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -5817,7 +5834,17 @@
 </file>
 
 <file path=xl/tables/table32.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D32" displayName="Table_TODO" name="Table_TODO" id="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B3" displayName="Table_Animations" name="Table_Animations" id="32">
+  <tableColumns count="2">
+    <tableColumn name="N" id="1"/>
+    <tableColumn name="ANIMATION_ID" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="ANIMATIONS-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D32" displayName="Table_TODO" name="Table_TODO" id="33">
   <tableColumns count="4">
     <tableColumn name="TASK" id="1"/>
     <tableColumn name="PRIO" id="2"/>
@@ -12843,6 +12870,51 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
+    <tabColor rgb="FF6FA8DC"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="19.0"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1319</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="36">
+        <f>ROW()-ROW(Table_Animations[N])</f>
+        <v>0</v>
+      </c>
+      <c r="B2" s="36" t="s">
+        <v>1361</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="36">
+        <f>ROW()-ROW(Table_Animations[N])</f>
+        <v>1</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>1362</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
@@ -12855,21 +12927,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1361</v>
+        <v>1363</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1362</v>
+        <v>1364</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="36" t="s">
-        <v>1365</v>
+        <v>1367</v>
       </c>
       <c r="B2" s="71">
         <v>1.0</v>
@@ -12883,7 +12955,7 @@
     </row>
     <row r="3">
       <c r="A3" s="36" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="B3" s="71">
         <v>1.0</v>
@@ -12897,7 +12969,7 @@
     </row>
     <row r="4">
       <c r="A4" s="36" t="s">
-        <v>1367</v>
+        <v>1369</v>
       </c>
       <c r="B4" s="71">
         <v>3.0</v>
@@ -12911,7 +12983,7 @@
     </row>
     <row r="5">
       <c r="A5" s="36" t="s">
-        <v>1368</v>
+        <v>1370</v>
       </c>
       <c r="B5" s="71">
         <v>1.0</v>
@@ -12925,7 +12997,7 @@
     </row>
     <row r="6">
       <c r="A6" s="36" t="s">
-        <v>1369</v>
+        <v>1371</v>
       </c>
       <c r="B6" s="71">
         <v>3.0</v>
@@ -12939,7 +13011,7 @@
     </row>
     <row r="7">
       <c r="A7" s="36" t="s">
-        <v>1370</v>
+        <v>1372</v>
       </c>
       <c r="B7" s="71">
         <v>3.0</v>
@@ -12953,7 +13025,7 @@
     </row>
     <row r="8">
       <c r="A8" s="36" t="s">
-        <v>1371</v>
+        <v>1373</v>
       </c>
       <c r="B8" s="71">
         <v>5.0</v>
@@ -12967,7 +13039,7 @@
     </row>
     <row r="9">
       <c r="A9" s="36" t="s">
-        <v>1372</v>
+        <v>1374</v>
       </c>
       <c r="B9" s="71">
         <v>4.0</v>
@@ -12981,7 +13053,7 @@
     </row>
     <row r="10">
       <c r="A10" s="36" t="s">
-        <v>1373</v>
+        <v>1375</v>
       </c>
       <c r="B10" s="71">
         <v>5.0</v>
@@ -12995,7 +13067,7 @@
     </row>
     <row r="11">
       <c r="A11" s="36" t="s">
-        <v>1374</v>
+        <v>1376</v>
       </c>
       <c r="B11" s="71">
         <v>4.0</v>
@@ -13009,7 +13081,7 @@
     </row>
     <row r="12">
       <c r="A12" s="36" t="s">
-        <v>1375</v>
+        <v>1377</v>
       </c>
       <c r="B12" s="71">
         <v>1.0</v>
@@ -13023,7 +13095,7 @@
     </row>
     <row r="13">
       <c r="A13" s="36" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
       <c r="B13" s="71">
         <v>4.0</v>
@@ -13037,7 +13109,7 @@
     </row>
     <row r="14">
       <c r="A14" s="36" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
       <c r="B14" s="71">
         <v>1.0</v>
@@ -13051,7 +13123,7 @@
     </row>
     <row r="15">
       <c r="A15" s="36" t="s">
-        <v>1378</v>
+        <v>1380</v>
       </c>
       <c r="B15" s="71">
         <v>2.0</v>
@@ -13065,7 +13137,7 @@
     </row>
     <row r="16">
       <c r="A16" s="36" t="s">
-        <v>1379</v>
+        <v>1381</v>
       </c>
       <c r="B16" s="71">
         <v>3.0</v>
@@ -13079,7 +13151,7 @@
     </row>
     <row r="17">
       <c r="A17" s="36" t="s">
-        <v>1380</v>
+        <v>1382</v>
       </c>
       <c r="B17" s="71">
         <v>2.0</v>
@@ -13093,7 +13165,7 @@
     </row>
     <row r="18">
       <c r="A18" s="36" t="s">
-        <v>1381</v>
+        <v>1383</v>
       </c>
       <c r="B18" s="71">
         <v>2.0</v>
@@ -13107,7 +13179,7 @@
     </row>
     <row r="19">
       <c r="A19" s="36" t="s">
-        <v>1382</v>
+        <v>1384</v>
       </c>
       <c r="B19" s="71">
         <v>2.0</v>
@@ -13121,7 +13193,7 @@
     </row>
     <row r="20">
       <c r="A20" s="36" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
       <c r="B20" s="71">
         <v>2.0</v>
@@ -13135,7 +13207,7 @@
     </row>
     <row r="21">
       <c r="A21" s="36" t="s">
-        <v>1384</v>
+        <v>1386</v>
       </c>
       <c r="B21" s="71">
         <v>3.0</v>
@@ -13149,7 +13221,7 @@
     </row>
     <row r="22">
       <c r="A22" s="36" t="s">
-        <v>1385</v>
+        <v>1387</v>
       </c>
       <c r="B22" s="71">
         <v>2.0</v>
@@ -13163,7 +13235,7 @@
     </row>
     <row r="23">
       <c r="A23" s="36" t="s">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="B23" s="71">
         <v>2.0</v>
@@ -13177,7 +13249,7 @@
     </row>
     <row r="24">
       <c r="A24" s="36" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="B24" s="71">
         <v>2.0</v>
@@ -13191,7 +13263,7 @@
     </row>
     <row r="25">
       <c r="A25" s="36" t="s">
-        <v>1388</v>
+        <v>1390</v>
       </c>
       <c r="B25" s="71">
         <v>2.0</v>
@@ -13205,7 +13277,7 @@
     </row>
     <row r="26">
       <c r="A26" s="36" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
       <c r="B26" s="71">
         <v>2.0</v>
@@ -13219,7 +13291,7 @@
     </row>
     <row r="27">
       <c r="A27" s="36" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="B27" s="71">
         <v>2.0</v>
@@ -13233,7 +13305,7 @@
     </row>
     <row r="28">
       <c r="A28" s="36" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="B28" s="71">
         <v>2.0</v>
@@ -13247,7 +13319,7 @@
     </row>
     <row r="29">
       <c r="A29" s="36" t="s">
-        <v>1392</v>
+        <v>1394</v>
       </c>
       <c r="B29" s="71">
         <v>4.0</v>
@@ -13261,7 +13333,7 @@
     </row>
     <row r="30">
       <c r="A30" s="36" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="B30" s="71">
         <v>2.0</v>
@@ -13275,7 +13347,7 @@
     </row>
     <row r="31">
       <c r="A31" s="36" t="s">
-        <v>1394</v>
+        <v>1396</v>
       </c>
       <c r="B31" s="71">
         <v>3.0</v>

</xml_diff>

<commit_message>
Character is loaded on each scene, but not included on each scene resources
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -11596,8 +11596,8 @@
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>1</v>
       </c>
-      <c r="B50" s="1" t="s">
-        <v>327</v>
+      <c r="B50" s="36" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="51">
@@ -11605,8 +11605,8 @@
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>2</v>
       </c>
-      <c r="B51" s="36" t="s">
-        <v>306</v>
+      <c r="B51" s="1" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="52">

</xml_diff>

<commit_message>
Fine tunning in scales in actual scenes
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -123,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4982" uniqueCount="1570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4982" uniqueCount="1571">
   <si>
     <t>NewItem</t>
   </si>
@@ -4563,6 +4563,9 @@
   </si>
   <si>
     <t>BACKGROUND_CITY1_SOUTH_STREET_1, BACKGROUND_CITY1_SOUTH_STREET_1_NIGHT</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_GENERIC_DOOR2</t>
   </si>
   <si>
     <t>CITY1_SOUTH_STREET_2</t>
@@ -10669,7 +10672,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="20.0"/>
+    <col customWidth="1" min="2" max="2" width="25.0"/>
     <col customWidth="1" min="3" max="3" width="45.71"/>
     <col customWidth="1" min="4" max="4" width="25.29"/>
     <col customWidth="1" min="5" max="5" width="41.71"/>
@@ -11060,7 +11063,7 @@
         <v>1479</v>
       </c>
       <c r="F12" s="35" t="s">
-        <v>325</v>
+        <v>1480</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>299</v>
@@ -11081,16 +11084,16 @@
         <v>10</v>
       </c>
       <c r="B13" s="29" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
       <c r="C13" s="32" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
       <c r="D13" s="34" t="s">
         <v>914</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
       <c r="F13" s="35" t="s">
         <v>325</v>
@@ -11117,13 +11120,13 @@
         <v>20</v>
       </c>
       <c r="C14" s="32" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="D14" s="34" t="s">
         <v>914</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="F14" s="35" t="s">
         <v>325</v>
@@ -11147,7 +11150,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="29" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
       <c r="C15" s="64" t="s">
         <v>301</v>
@@ -11210,7 +11213,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="2">
@@ -11237,7 +11240,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="5">
@@ -11246,7 +11249,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="36" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="6">
@@ -11258,7 +11261,7 @@
         <v>44</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="8">
@@ -11266,7 +11269,7 @@
         <v>0.0</v>
       </c>
       <c r="B8" s="36" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="9">
@@ -11274,7 +11277,7 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="36" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="10">
@@ -11282,7 +11285,7 @@
         <v>2.0</v>
       </c>
       <c r="B10" s="36" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="11">
@@ -11290,7 +11293,7 @@
         <v>3.0</v>
       </c>
       <c r="B11" s="36" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="12">
@@ -11298,7 +11301,7 @@
         <v>4.0</v>
       </c>
       <c r="B12" s="36" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="13">
@@ -11306,7 +11309,7 @@
         <v>5.0</v>
       </c>
       <c r="B13" s="36" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="15">
@@ -11314,7 +11317,7 @@
         <v>44</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="16">
@@ -11332,7 +11335,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="36" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="18">
@@ -11377,7 +11380,7 @@
         <v>6</v>
       </c>
       <c r="B22" s="36" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="23">
@@ -11403,7 +11406,7 @@
         <v>44</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="27">
@@ -11448,7 +11451,7 @@
         <v>4</v>
       </c>
       <c r="B31" s="36" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="32">
@@ -11475,7 +11478,7 @@
         <v>7</v>
       </c>
       <c r="B34" s="36" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="35">
@@ -11493,7 +11496,7 @@
         <v>9</v>
       </c>
       <c r="B36" s="36" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="37">
@@ -11555,7 +11558,7 @@
         <v>44</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="45">
@@ -11579,7 +11582,7 @@
         <v>44</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="49">
@@ -11632,7 +11635,7 @@
         <v>44</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="56">
@@ -11697,7 +11700,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="2">
@@ -11715,7 +11718,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="4">
@@ -11724,7 +11727,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="5">
@@ -11805,7 +11808,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="36" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="14">
@@ -11994,7 +11997,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="36" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="36">
@@ -12002,16 +12005,16 @@
         <v>44</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
       <c r="C36" s="66" t="s">
         <v>290</v>
       </c>
       <c r="D36" s="66" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="E36" s="66" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="37">
@@ -12020,7 +12023,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="36" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="C37" s="38" t="s">
         <v>299</v>
@@ -12039,7 +12042,7 @@
         <v>1</v>
       </c>
       <c r="B38" s="36" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="C38" s="38" t="s">
         <v>1057</v>
@@ -12058,7 +12061,7 @@
         <v>2</v>
       </c>
       <c r="B39" s="36" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="C39" s="38" t="s">
         <v>1088</v>
@@ -12096,7 +12099,7 @@
         <v>4</v>
       </c>
       <c r="B41" s="36" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="C41" s="38" t="s">
         <v>427</v>
@@ -12114,19 +12117,19 @@
         <v>44</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="C43" s="65" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="D43" s="65" t="s">
         <v>1020</v>
       </c>
       <c r="E43" s="66" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="F43" s="65" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="44">
@@ -12138,13 +12141,13 @@
         <v>670</v>
       </c>
       <c r="C44" s="44" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="D44" s="44" t="s">
         <v>673</v>
       </c>
       <c r="E44" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F44" s="43" t="b">
         <v>0</v>
@@ -12159,13 +12162,13 @@
         <v>682</v>
       </c>
       <c r="C45" s="44" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="D45" s="44" t="s">
         <v>1164</v>
       </c>
       <c r="E45" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F45" s="43" t="b">
         <v>0</v>
@@ -12180,13 +12183,13 @@
         <v>699</v>
       </c>
       <c r="C46" s="44" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="D46" s="44" t="s">
         <v>719</v>
       </c>
       <c r="E46" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F46" s="43" t="b">
         <v>0</v>
@@ -12201,13 +12204,13 @@
         <v>704</v>
       </c>
       <c r="C47" s="44" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="D47" s="44" t="s">
         <v>1266</v>
       </c>
       <c r="E47" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F47" s="43" t="b">
         <v>0</v>
@@ -12228,7 +12231,7 @@
         <v>1339</v>
       </c>
       <c r="E48" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F48" s="43" t="b">
         <v>0</v>
@@ -12240,7 +12243,7 @@
         <v>5</v>
       </c>
       <c r="B49" s="36" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
       <c r="C49" s="44" t="s">
         <v>39</v>
@@ -12249,7 +12252,7 @@
         <v>1342</v>
       </c>
       <c r="E49" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F49" s="43" t="b">
         <v>0</v>
@@ -12261,7 +12264,7 @@
         <v>6</v>
       </c>
       <c r="B50" s="36" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="C50" s="44" t="s">
         <v>39</v>
@@ -12270,7 +12273,7 @@
         <v>1345</v>
       </c>
       <c r="E50" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F50" s="43" t="b">
         <v>1</v>
@@ -12282,16 +12285,16 @@
         <v>7</v>
       </c>
       <c r="B51" s="36" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="C51" s="44" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="D51" s="44" t="s">
         <v>673</v>
       </c>
       <c r="E51" s="48" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="F51" s="43" t="b">
         <v>0</v>
@@ -12302,10 +12305,10 @@
         <v>44</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="C53" s="28" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="54">
@@ -12314,7 +12317,7 @@
         <v>0</v>
       </c>
       <c r="B54" s="36" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="C54" s="51" t="s">
         <v>436</v>
@@ -12325,7 +12328,7 @@
         <v>44</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="57">
@@ -13335,16 +13338,16 @@
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="2">
@@ -13356,7 +13359,7 @@
         <v>302</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="D2" s="68" t="s">
         <v>299</v>
@@ -13374,7 +13377,7 @@
         <v>417</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>299</v>
@@ -13389,10 +13392,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="D4" s="68" t="s">
         <v>299</v>
@@ -13430,7 +13433,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
     </row>
     <row r="2">
@@ -13457,7 +13460,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
     </row>
   </sheetData>
@@ -13483,21 +13486,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="37" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="B2" s="69">
         <v>1.0</v>
@@ -13511,7 +13514,7 @@
     </row>
     <row r="3">
       <c r="A3" s="37" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
       <c r="B3" s="69">
         <v>1.0</v>
@@ -13525,7 +13528,7 @@
     </row>
     <row r="4">
       <c r="A4" s="37" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="B4" s="69">
         <v>3.0</v>
@@ -13539,7 +13542,7 @@
     </row>
     <row r="5">
       <c r="A5" s="37" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="B5" s="69">
         <v>1.0</v>
@@ -13553,7 +13556,7 @@
     </row>
     <row r="6">
       <c r="A6" s="37" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="B6" s="69">
         <v>3.0</v>
@@ -13567,7 +13570,7 @@
     </row>
     <row r="7">
       <c r="A7" s="37" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="B7" s="69">
         <v>3.0</v>
@@ -13581,7 +13584,7 @@
     </row>
     <row r="8">
       <c r="A8" s="37" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="B8" s="69">
         <v>5.0</v>
@@ -13595,7 +13598,7 @@
     </row>
     <row r="9">
       <c r="A9" s="37" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="B9" s="69">
         <v>4.0</v>
@@ -13609,7 +13612,7 @@
     </row>
     <row r="10">
       <c r="A10" s="37" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="B10" s="69">
         <v>5.0</v>
@@ -13623,7 +13626,7 @@
     </row>
     <row r="11">
       <c r="A11" s="37" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="B11" s="69">
         <v>4.0</v>
@@ -13637,7 +13640,7 @@
     </row>
     <row r="12">
       <c r="A12" s="37" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="B12" s="69">
         <v>1.0</v>
@@ -13651,7 +13654,7 @@
     </row>
     <row r="13">
       <c r="A13" s="37" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="B13" s="69">
         <v>4.0</v>
@@ -13665,7 +13668,7 @@
     </row>
     <row r="14">
       <c r="A14" s="37" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="B14" s="69">
         <v>1.0</v>
@@ -13679,7 +13682,7 @@
     </row>
     <row r="15">
       <c r="A15" s="37" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
       <c r="B15" s="69">
         <v>2.0</v>
@@ -13693,7 +13696,7 @@
     </row>
     <row r="16">
       <c r="A16" s="37" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="B16" s="69">
         <v>3.0</v>
@@ -13707,7 +13710,7 @@
     </row>
     <row r="17">
       <c r="A17" s="37" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="B17" s="69">
         <v>2.0</v>
@@ -13721,7 +13724,7 @@
     </row>
     <row r="18">
       <c r="A18" s="37" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="B18" s="69">
         <v>2.0</v>
@@ -13735,7 +13738,7 @@
     </row>
     <row r="19">
       <c r="A19" s="37" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="B19" s="69">
         <v>2.0</v>
@@ -13749,7 +13752,7 @@
     </row>
     <row r="20">
       <c r="A20" s="37" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="B20" s="69">
         <v>2.0</v>
@@ -13763,7 +13766,7 @@
     </row>
     <row r="21">
       <c r="A21" s="37" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="B21" s="69">
         <v>3.0</v>
@@ -13777,7 +13780,7 @@
     </row>
     <row r="22">
       <c r="A22" s="37" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="B22" s="69">
         <v>2.0</v>
@@ -13791,7 +13794,7 @@
     </row>
     <row r="23">
       <c r="A23" s="37" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="B23" s="69">
         <v>2.0</v>
@@ -13805,7 +13808,7 @@
     </row>
     <row r="24">
       <c r="A24" s="37" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="B24" s="69">
         <v>2.0</v>
@@ -13819,7 +13822,7 @@
     </row>
     <row r="25">
       <c r="A25" s="37" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="B25" s="69">
         <v>2.0</v>
@@ -13833,7 +13836,7 @@
     </row>
     <row r="26">
       <c r="A26" s="37" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="B26" s="69">
         <v>2.0</v>
@@ -13847,7 +13850,7 @@
     </row>
     <row r="27">
       <c r="A27" s="37" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="B27" s="69">
         <v>2.0</v>
@@ -13861,7 +13864,7 @@
     </row>
     <row r="28">
       <c r="A28" s="37" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="B28" s="69">
         <v>2.0</v>
@@ -13875,7 +13878,7 @@
     </row>
     <row r="29">
       <c r="A29" s="37" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="B29" s="69">
         <v>4.0</v>
@@ -13889,7 +13892,7 @@
     </row>
     <row r="30">
       <c r="A30" s="37" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="B30" s="69">
         <v>2.0</v>
@@ -13903,7 +13906,7 @@
     </row>
     <row r="31">
       <c r="A31" s="37" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="B31" s="69">
         <v>3.0</v>
@@ -13917,7 +13920,7 @@
     </row>
     <row r="32">
       <c r="A32" s="37" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="B32" s="69">
         <v>2.0</v>

</xml_diff>

<commit_message>
[Partial] Fading between scenes
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -101,32 +101,8 @@
 </comments>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
-  <authors>
-    <author/>
-  </authors>
-  <commentList>
-    <comment authorId="0" ref="A20">
-      <text>
-        <t xml:space="preserve">NullReferenceException: Object reference not set to an instance of an object
-Gob3AQ.GameMenu.Dialog.DialogOptionButtonClass.SetOptionText (System.String&amp; text) (at Assets/Scripts/Menu/DialogOptionButtonClass.cs:27)
-Gob3AQ.GameMenu.GameMenuClass.ShowDialogueService (System.ReadOnlySpan`1[T] defaultTalkers, Gob3AQ.VARMAP.Types.DialogType dialog, Gob3AQ.VARMAP.Types.DialogPhrase phrase) (at Assets/Scripts/Master/GameMenuClass.cs:93)
-Gob3AQ.GameMaster.GameMasterClass.EnableDialogueService (System.Boolean enable, System.ReadOnlySpan`1[T] talkers, Gob3AQ.VARMAP.Types.DialogType dialog, Gob3AQ.VARMAP.Types.DialogPhrase phrase) (at Assets/Scripts/Master/GameMasterClass.cs:232)
-Gob3AQ.LevelMaster.LevelMasterClass.PlayerReachedWaypointService (Gob3AQ.VARMAP.Types.CharacterType character) (at Assets/Scripts/Master/LevelMasterClass.cs:183)
-Gob3AQ.GameElement.PlayableChar.PlayableCharScript.StartBufferedInteraction () (at Assets/Scripts/GameElement/PlayableCharScript.cs:351)
-Gob3AQ.GameElement.PlayableChar.PlayableCharScript.Execute_Walk () (at Assets/Scripts/GameElement/PlayableCharScript.cs:279)
-Gob3AQ.GameElement.PlayableChar.PlayableCharScript.Execute_Play () (at Assets/Scripts/GameElement/PlayableCharScript.cs:234)
-Gob3AQ.GameElement.PlayableChar.PlayableCharScript.Update () (at Assets/Scripts/GameElement/PlayableCharScript.cs:164)
-</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5035" uniqueCount="1590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5011" uniqueCount="1566">
   <si>
     <t>NewItem</t>
   </si>
@@ -4805,97 +4781,25 @@
     <t>ONGOING</t>
   </si>
   <si>
-    <t>Talk with characters</t>
-  </si>
-  <si>
-    <t>Plot (1st part)</t>
-  </si>
-  <si>
-    <t>Improve Waypoint Tool (naming)</t>
-  </si>
-  <si>
-    <t>Language files</t>
-  </si>
-  <si>
-    <t>Background objects layers</t>
-  </si>
-  <si>
-    <t>Bug with menu of items (not selecting)</t>
-  </si>
-  <si>
-    <t>Loading screen between rooms</t>
-  </si>
-  <si>
-    <t>Main event list (Tomba style)</t>
-  </si>
-  <si>
     <t>Parry - Notifications - Max 4 queue</t>
   </si>
   <si>
     <t>Trophies</t>
   </si>
   <si>
-    <t>Observe items, NPCs, trigger events</t>
-  </si>
-  <si>
-    <t>Seealso in services. Add owner in descr</t>
-  </si>
-  <si>
-    <t>Avoid services modifying VARMAP</t>
-  </si>
-  <si>
-    <t>Normalize menu items with dialog opts</t>
-  </si>
-  <si>
-    <t>Use Dictionaries for LevelManager</t>
-  </si>
-  <si>
-    <t>State change deactivation/activation</t>
-  </si>
-  <si>
-    <t>Adressables instead of Resources</t>
-  </si>
-  <si>
-    <t>Sprite Atlas addressable</t>
-  </si>
-  <si>
-    <t>Enshorten stack</t>
-  </si>
-  <si>
-    <t>Re-think usage of ITEM_TAKE, USE_TALK</t>
-  </si>
-  <si>
-    <t>Spawn/Despawn conditions</t>
-  </si>
-  <si>
-    <t>Drag with mouse</t>
-  </si>
-  <si>
-    <t>Zoom</t>
-  </si>
-  <si>
-    <t>More upper button commands</t>
-  </si>
-  <si>
-    <t>Waypoint numeration in Editor</t>
-  </si>
-  <si>
-    <t>Use one raycast for all objets (Input)</t>
-  </si>
-  <si>
-    <t>Make character go slower on far depths</t>
-  </si>
-  <si>
     <t>Waypoints only reachable for actions</t>
   </si>
   <si>
-    <t>Decission actions (like dialogs)</t>
-  </si>
-  <si>
     <t>Reduce cond stackallocs (they use JIT)</t>
   </si>
   <si>
-    <t>If you click on player many times when he's facing to a door it appears unselected in next room</t>
+    <t>Character 'Señor desubicado'</t>
+  </si>
+  <si>
+    <t>Questioning 'Mosca puñetera'</t>
+  </si>
+  <si>
+    <t>Fade to black between scenes</t>
   </si>
 </sst>
 </file>
@@ -6452,7 +6356,7 @@
 </file>
 
 <file path=xl/tables/table34.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D33" displayName="Table_TODO" name="Table_TODO" id="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D9" displayName="Table_TODO" name="Table_TODO" id="34">
   <tableColumns count="4">
     <tableColumn name="TASK" id="1"/>
     <tableColumn name="PRIO" id="2"/>
@@ -13585,13 +13489,13 @@
         <v>1559</v>
       </c>
       <c r="B2" s="70">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="C2" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -13599,13 +13503,13 @@
         <v>1560</v>
       </c>
       <c r="B3" s="70">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="C3" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -13613,13 +13517,13 @@
         <v>1561</v>
       </c>
       <c r="B4" s="70">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="C4" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -13627,13 +13531,13 @@
         <v>1562</v>
       </c>
       <c r="B5" s="70">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="C5" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -13641,13 +13545,13 @@
         <v>1563</v>
       </c>
       <c r="B6" s="70">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C6" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -13655,13 +13559,13 @@
         <v>1564</v>
       </c>
       <c r="B7" s="70">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C7" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -13669,10 +13573,10 @@
         <v>1565</v>
       </c>
       <c r="B8" s="70">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="C8" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="36" t="b">
         <v>1</v>
@@ -13680,356 +13584,20 @@
     </row>
     <row r="9">
       <c r="A9" s="37" t="s">
-        <v>1566</v>
+        <v>1131</v>
       </c>
       <c r="B9" s="70">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="C9" s="36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="37" t="s">
-        <v>1567</v>
-      </c>
-      <c r="B10" s="70">
-        <v>5.0</v>
-      </c>
-      <c r="C10" s="36" t="b">
         <v>0</v>
       </c>
-      <c r="D10" s="36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="37" t="s">
-        <v>1568</v>
-      </c>
-      <c r="B11" s="70">
-        <v>4.0</v>
-      </c>
-      <c r="C11" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="D11" s="36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="37" t="s">
-        <v>1569</v>
-      </c>
-      <c r="B12" s="70">
-        <v>1.0</v>
-      </c>
-      <c r="C12" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="37" t="s">
-        <v>1570</v>
-      </c>
-      <c r="B13" s="70">
-        <v>4.0</v>
-      </c>
-      <c r="C13" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="37" t="s">
-        <v>1571</v>
-      </c>
-      <c r="B14" s="70">
-        <v>1.0</v>
-      </c>
-      <c r="C14" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="37" t="s">
-        <v>1572</v>
-      </c>
-      <c r="B15" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C15" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D15" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="37" t="s">
-        <v>1573</v>
-      </c>
-      <c r="B16" s="70">
-        <v>3.0</v>
-      </c>
-      <c r="C16" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D16" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="37" t="s">
-        <v>1574</v>
-      </c>
-      <c r="B17" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C17" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D17" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="37" t="s">
-        <v>1575</v>
-      </c>
-      <c r="B18" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C18" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D18" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="37" t="s">
-        <v>1576</v>
-      </c>
-      <c r="B19" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C19" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D19" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="37" t="s">
-        <v>1577</v>
-      </c>
-      <c r="B20" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C20" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D20" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="37" t="s">
-        <v>1578</v>
-      </c>
-      <c r="B21" s="70">
-        <v>3.0</v>
-      </c>
-      <c r="C21" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D21" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="37" t="s">
-        <v>1579</v>
-      </c>
-      <c r="B22" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C22" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D22" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="37" t="s">
-        <v>1580</v>
-      </c>
-      <c r="B23" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C23" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D23" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="37" t="s">
-        <v>1581</v>
-      </c>
-      <c r="B24" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C24" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D24" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="37" t="s">
-        <v>1582</v>
-      </c>
-      <c r="B25" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C25" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D25" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="37" t="s">
-        <v>1583</v>
-      </c>
-      <c r="B26" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C26" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D26" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="37" t="s">
-        <v>1584</v>
-      </c>
-      <c r="B27" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C27" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D27" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="37" t="s">
-        <v>1585</v>
-      </c>
-      <c r="B28" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C28" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D28" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="37" t="s">
-        <v>1586</v>
-      </c>
-      <c r="B29" s="70">
-        <v>4.0</v>
-      </c>
-      <c r="C29" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="D29" s="36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="37" t="s">
-        <v>1587</v>
-      </c>
-      <c r="B30" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C30" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D30" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="37" t="s">
-        <v>1588</v>
-      </c>
-      <c r="B31" s="70">
-        <v>3.0</v>
-      </c>
-      <c r="C31" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="D31" s="36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="37" t="s">
-        <v>1589</v>
-      </c>
-      <c r="B32" s="70">
-        <v>2.0</v>
-      </c>
-      <c r="C32" s="36" t="b">
-        <v>1</v>
-      </c>
-      <c r="D32" s="36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="37" t="s">
-        <v>1131</v>
-      </c>
-      <c r="B33" s="70">
-        <v>5.0</v>
-      </c>
-      <c r="C33" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="D33" s="36" t="b">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B33">
+  <conditionalFormatting sqref="B2:B9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="formula" val="1"/>
@@ -14041,20 +13609,19 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A33">
+  <conditionalFormatting sqref="A2:A9">
     <cfRule type="expression" dxfId="5" priority="2">
       <formula>$C2=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="B2:B33">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="B2:B9">
       <formula1>AND(ISNUMBER(B2),(NOT(OR(NOT(ISERROR(DATEVALUE(B2))), AND(ISNUMBER(B2), LEFT(CELL("format", B2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Starting with dialog animations
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5117" uniqueCount="1570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5131" uniqueCount="1584">
   <si>
     <t>NewItem</t>
   </si>
@@ -3518,7 +3518,7 @@
     <t>Sound</t>
   </si>
   <si>
-    <t>CharAnimation</t>
+    <t>AnimationTrigger</t>
   </si>
   <si>
     <t>Text_English</t>
@@ -3527,10 +3527,10 @@
     <t>Text_Spanish</t>
   </si>
   <si>
-    <t>DIALOG_ANIMATION_NONE</t>
-  </si>
-  <si>
-    <t>DIALOG_ANIMATION_TALK</t>
+    <t>ANIMATION_TRIGGER_NONE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_TALK</t>
   </si>
   <si>
     <t>That has no sense!</t>
@@ -4676,7 +4676,49 @@
     <t>ACTION_TYPE_NOTIF</t>
   </si>
   <si>
-    <t>DIALOG_ANIMATION_ID</t>
+    <t>ANIMATION_TRIGGER_ID</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_ONE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_TWO</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_THREE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_FOUR</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_FIVE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_SIX</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_SPECIAL_ONE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_SPECIAL_TWO</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_STEADY</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_WALK_FRONT</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_WALK_BACK</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_WALK_CORNERBACK</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_WALK_CORNERFRONT</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_WALK_SIDE</t>
   </si>
   <si>
     <t>ITEM_FAMILY_TYPE_ID</t>
@@ -6164,7 +6206,7 @@
     <tableColumn name="PHRASE_ID" id="2"/>
     <tableColumn name="TalkerIndex" id="3"/>
     <tableColumn name="Sound" id="4"/>
-    <tableColumn name="CharAnimation" id="5"/>
+    <tableColumn name="AnimationTrigger" id="5"/>
     <tableColumn name="Text_English" id="6"/>
     <tableColumn name="Text_Spanish" id="7"/>
   </tableColumns>
@@ -6245,17 +6287,17 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A43:B45" displayName="Table_Dialog_Animation" name="Table_Dialog_Animation" id="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A43:B59" displayName="Table_Animation_Trigger" name="Table_Animation_Trigger" id="24">
   <tableColumns count="2">
     <tableColumn name="N" id="1"/>
-    <tableColumn name="DIALOG_ANIMATION_ID" id="2"/>
+    <tableColumn name="ANIMATION_TRIGGER_ID" id="2"/>
   </tableColumns>
   <tableStyleInfo name="TYPES-style 5" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A47:B52" displayName="Table_Item_Family_Type" name="Table_Item_Family_Type" id="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A61:B66" displayName="Table_Item_Family_Type" name="Table_Item_Family_Type" id="25">
   <tableColumns count="2">
     <tableColumn name="N" id="1"/>
     <tableColumn name="ITEM_FAMILY_TYPE_ID" id="2"/>
@@ -6265,7 +6307,7 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A54:B57" displayName="Table_Moment_Day" name="Table_Moment_Day" id="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A68:B71" displayName="Table_Moment_Day" name="Table_Moment_Day" id="26">
   <tableColumns count="2">
     <tableColumn name="N" id="1"/>
     <tableColumn name="MOMENT_TYPE_ID" id="2"/>
@@ -7605,7 +7647,7 @@
     <col customWidth="1" min="2" max="2" width="65.43"/>
     <col customWidth="1" min="3" max="3" width="15.57"/>
     <col customWidth="1" min="4" max="4" width="26.86"/>
-    <col customWidth="1" min="5" max="5" width="32.86"/>
+    <col customWidth="1" min="5" max="5" width="34.14"/>
     <col customWidth="1" min="6" max="6" width="50.29"/>
     <col customWidth="1" min="7" max="7" width="58.43"/>
     <col customWidth="1" min="8" max="8" width="32.86"/>
@@ -10657,10 +10699,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="E2:E127">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D127">
+    <dataValidation type="list" allowBlank="1" sqref="D2:E127">
       <formula1>#REF!</formula1>
     </dataValidation>
   </dataValidations>
@@ -11252,7 +11291,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="40.29"/>
+    <col customWidth="1" min="2" max="2" width="44.0"/>
     <col customWidth="1" min="3" max="3" width="38.86"/>
     <col customWidth="1" min="4" max="4" width="23.29"/>
     <col customWidth="1" min="6" max="6" width="38.86"/>
@@ -11605,7 +11644,8 @@
     </row>
     <row r="44">
       <c r="A44" s="36">
-        <v>0.0</v>
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>0</v>
       </c>
       <c r="B44" s="36" t="s">
         <v>1141</v>
@@ -11613,97 +11653,224 @@
     </row>
     <row r="45">
       <c r="A45" s="36">
-        <v>1.0</v>
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>1</v>
       </c>
       <c r="B45" s="36" t="s">
-        <v>1142</v>
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>2</v>
+      </c>
+      <c r="B46" s="36" t="s">
+        <v>1526</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>1525</v>
+      <c r="A47" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>3</v>
+      </c>
+      <c r="B47" s="36" t="s">
+        <v>1527</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="36">
-        <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
-        <v>0</v>
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>4</v>
       </c>
       <c r="B48" s="36" t="s">
-        <v>311</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>5</v>
+      </c>
+      <c r="B49" s="36" t="s">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>6</v>
+      </c>
+      <c r="B50" s="36" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>7</v>
+      </c>
+      <c r="B51" s="36" t="s">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>8</v>
+      </c>
+      <c r="B52" s="36" t="s">
+        <v>1532</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>9</v>
+      </c>
+      <c r="B53" s="36" t="s">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>10</v>
+      </c>
+      <c r="B54" s="36" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>11</v>
+      </c>
+      <c r="B55" s="36" t="s">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>12</v>
+      </c>
+      <c r="B56" s="36" t="s">
+        <v>1535</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>13</v>
+      </c>
+      <c r="B57" s="36" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>14</v>
+      </c>
+      <c r="B58" s="36" t="s">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="36">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>15</v>
+      </c>
+      <c r="B59" s="36" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="36">
+        <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
+        <v>0</v>
+      </c>
+      <c r="B62" s="36" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="36">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>1</v>
       </c>
-      <c r="B49" s="36" t="s">
+      <c r="B63" s="36" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="36">
+    <row r="64">
+      <c r="A64" s="36">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>2</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B64" s="1" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="36">
+    <row r="65">
+      <c r="A65" s="36">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>3</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B65" s="1" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="36">
+    <row r="66">
+      <c r="A66" s="36">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>4</v>
       </c>
-      <c r="B52" s="67" t="s">
+      <c r="B66" s="67" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="1" t="s">
+    <row r="68">
+      <c r="A68" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>1526</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="36">
+      <c r="B68" s="1" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="36">
         <f>ROW()-ROW(Table_Moment_Day[N])</f>
         <v>0</v>
       </c>
-      <c r="B55" s="36" t="s">
+      <c r="B69" s="36" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="36">
+    <row r="70">
+      <c r="A70" s="36">
         <f>ROW()-ROW(Table_Moment_Day[N])</f>
         <v>1</v>
       </c>
-      <c r="B56" s="36" t="s">
+      <c r="B70" s="36" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="36">
+    <row r="71">
+      <c r="A71" s="36">
         <f>ROW()-ROW(Table_Moment_Day[N])</f>
         <v>2</v>
       </c>
-      <c r="B57" s="36" t="s">
+      <c r="B71" s="36" t="s">
         <v>451</v>
       </c>
     </row>
@@ -11742,7 +11909,7 @@
         <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1527</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="2">
@@ -11760,7 +11927,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>1528</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="4">
@@ -11769,7 +11936,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1529</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="5">
@@ -11850,7 +12017,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="36" t="s">
-        <v>1530</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="14">
@@ -11895,7 +12062,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="36" t="s">
-        <v>1531</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="19">
@@ -12039,7 +12206,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="36" t="s">
-        <v>1532</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="36">
@@ -12047,16 +12214,16 @@
         <v>46</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>1533</v>
+        <v>1547</v>
       </c>
       <c r="C36" s="68" t="s">
         <v>301</v>
       </c>
       <c r="D36" s="68" t="s">
-        <v>1534</v>
+        <v>1548</v>
       </c>
       <c r="E36" s="68" t="s">
-        <v>1535</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="37">
@@ -12065,7 +12232,7 @@
         <v>0</v>
       </c>
       <c r="B37" s="36" t="s">
-        <v>1536</v>
+        <v>1550</v>
       </c>
       <c r="C37" s="38" t="s">
         <v>310</v>
@@ -12084,7 +12251,7 @@
         <v>1</v>
       </c>
       <c r="B38" s="36" t="s">
-        <v>1537</v>
+        <v>1551</v>
       </c>
       <c r="C38" s="38" t="s">
         <v>1074</v>
@@ -12103,7 +12270,7 @@
         <v>2</v>
       </c>
       <c r="B39" s="36" t="s">
-        <v>1538</v>
+        <v>1552</v>
       </c>
       <c r="C39" s="38" t="s">
         <v>1105</v>
@@ -12141,7 +12308,7 @@
         <v>4</v>
       </c>
       <c r="B41" s="36" t="s">
-        <v>1539</v>
+        <v>1553</v>
       </c>
       <c r="C41" s="38" t="s">
         <v>441</v>
@@ -12159,19 +12326,19 @@
         <v>46</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>1540</v>
+        <v>1554</v>
       </c>
       <c r="C43" s="67" t="s">
-        <v>1541</v>
+        <v>1555</v>
       </c>
       <c r="D43" s="67" t="s">
         <v>1037</v>
       </c>
       <c r="E43" s="68" t="s">
-        <v>1542</v>
+        <v>1556</v>
       </c>
       <c r="F43" s="67" t="s">
-        <v>1543</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="44">
@@ -12183,13 +12350,13 @@
         <v>686</v>
       </c>
       <c r="C44" s="44" t="s">
-        <v>1536</v>
+        <v>1550</v>
       </c>
       <c r="D44" s="44" t="s">
         <v>689</v>
       </c>
       <c r="E44" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F44" s="43" t="b">
         <v>0</v>
@@ -12204,13 +12371,13 @@
         <v>698</v>
       </c>
       <c r="C45" s="44" t="s">
-        <v>1537</v>
+        <v>1551</v>
       </c>
       <c r="D45" s="44" t="s">
         <v>1182</v>
       </c>
       <c r="E45" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F45" s="43" t="b">
         <v>0</v>
@@ -12225,13 +12392,13 @@
         <v>715</v>
       </c>
       <c r="C46" s="44" t="s">
-        <v>1537</v>
+        <v>1551</v>
       </c>
       <c r="D46" s="44" t="s">
         <v>735</v>
       </c>
       <c r="E46" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F46" s="43" t="b">
         <v>0</v>
@@ -12246,13 +12413,13 @@
         <v>720</v>
       </c>
       <c r="C47" s="44" t="s">
-        <v>1538</v>
+        <v>1552</v>
       </c>
       <c r="D47" s="44" t="s">
         <v>1284</v>
       </c>
       <c r="E47" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F47" s="43" t="b">
         <v>0</v>
@@ -12273,7 +12440,7 @@
         <v>1357</v>
       </c>
       <c r="E48" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F48" s="43" t="b">
         <v>0</v>
@@ -12285,7 +12452,7 @@
         <v>5</v>
       </c>
       <c r="B49" s="36" t="s">
-        <v>1545</v>
+        <v>1559</v>
       </c>
       <c r="C49" s="44" t="s">
         <v>41</v>
@@ -12294,7 +12461,7 @@
         <v>1360</v>
       </c>
       <c r="E49" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F49" s="43" t="b">
         <v>0</v>
@@ -12306,7 +12473,7 @@
         <v>6</v>
       </c>
       <c r="B50" s="36" t="s">
-        <v>1546</v>
+        <v>1560</v>
       </c>
       <c r="C50" s="44" t="s">
         <v>41</v>
@@ -12315,7 +12482,7 @@
         <v>1363</v>
       </c>
       <c r="E50" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F50" s="43" t="b">
         <v>1</v>
@@ -12327,16 +12494,16 @@
         <v>7</v>
       </c>
       <c r="B51" s="36" t="s">
-        <v>1547</v>
+        <v>1561</v>
       </c>
       <c r="C51" s="44" t="s">
-        <v>1539</v>
+        <v>1553</v>
       </c>
       <c r="D51" s="44" t="s">
         <v>689</v>
       </c>
       <c r="E51" s="48" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="F51" s="43" t="b">
         <v>0</v>
@@ -12347,10 +12514,10 @@
         <v>46</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>1548</v>
+        <v>1562</v>
       </c>
       <c r="C53" s="28" t="s">
-        <v>1549</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="54">
@@ -12359,7 +12526,7 @@
         <v>0</v>
       </c>
       <c r="B54" s="36" t="s">
-        <v>1544</v>
+        <v>1558</v>
       </c>
       <c r="C54" s="51" t="s">
         <v>450</v>
@@ -12370,7 +12537,7 @@
         <v>46</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>1550</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="57">
@@ -13380,16 +13547,16 @@
         <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1551</v>
+        <v>1565</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1552</v>
+        <v>1566</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1553</v>
+        <v>1567</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1554</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="2">
@@ -13401,7 +13568,7 @@
         <v>313</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>1555</v>
+        <v>1569</v>
       </c>
       <c r="D2" s="70" t="s">
         <v>310</v>
@@ -13419,7 +13586,7 @@
         <v>428</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>1556</v>
+        <v>1570</v>
       </c>
       <c r="D3" s="70" t="s">
         <v>310</v>
@@ -13434,10 +13601,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="29" t="s">
-        <v>1557</v>
+        <v>1571</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>1555</v>
+        <v>1569</v>
       </c>
       <c r="D4" s="70" t="s">
         <v>310</v>
@@ -13502,7 +13669,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="36" t="s">
-        <v>1558</v>
+        <v>1572</v>
       </c>
     </row>
   </sheetData>
@@ -13528,21 +13695,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1559</v>
+        <v>1573</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1560</v>
+        <v>1574</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1561</v>
+        <v>1575</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1562</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="37" t="s">
-        <v>1563</v>
+        <v>1577</v>
       </c>
       <c r="B2" s="71">
         <v>5.0</v>
@@ -13556,7 +13723,7 @@
     </row>
     <row r="3">
       <c r="A3" s="37" t="s">
-        <v>1564</v>
+        <v>1578</v>
       </c>
       <c r="B3" s="71">
         <v>4.0</v>
@@ -13570,7 +13737,7 @@
     </row>
     <row r="4">
       <c r="A4" s="37" t="s">
-        <v>1565</v>
+        <v>1579</v>
       </c>
       <c r="B4" s="71">
         <v>2.0</v>
@@ -13584,7 +13751,7 @@
     </row>
     <row r="5">
       <c r="A5" s="37" t="s">
-        <v>1566</v>
+        <v>1580</v>
       </c>
       <c r="B5" s="71">
         <v>5.0</v>
@@ -13598,7 +13765,7 @@
     </row>
     <row r="6">
       <c r="A6" s="37" t="s">
-        <v>1567</v>
+        <v>1581</v>
       </c>
       <c r="B6" s="71">
         <v>4.0</v>
@@ -13612,7 +13779,7 @@
     </row>
     <row r="7">
       <c r="A7" s="37" t="s">
-        <v>1568</v>
+        <v>1582</v>
       </c>
       <c r="B7" s="71">
         <v>4.0</v>
@@ -13626,7 +13793,7 @@
     </row>
     <row r="8">
       <c r="A8" s="37" t="s">
-        <v>1569</v>
+        <v>1583</v>
       </c>
       <c r="B8" s="71">
         <v>2.0</v>

</xml_diff>

<commit_message>
Fire and avoided Action selector showing between scenes
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -2219,13 +2219,13 @@
     <t>UNCHAIN_EXTRAPERLO_DOOR</t>
   </si>
   <si>
+    <t>ACTION_SPAWN_EXTRAPERLO_DOOR</t>
+  </si>
+  <si>
+    <t>UNCHAIN_SHOW_EXTRAPERLO_DOOR_OPENED</t>
+  </si>
+  <si>
     <t>EVENT_EXTRAPERLO_SAID_PHRASE</t>
-  </si>
-  <si>
-    <t>ACTION_SPAWN_EXTRAPERLO_DOOR</t>
-  </si>
-  <si>
-    <t>UNCHAIN_SHOW_EXTRAPERLO_DOOR_OPENED</t>
   </si>
   <si>
     <t>ACTION_SPAWN_EXTRAPERLO_WALL, ACTION_DESPAWN_EXTRAPERLO_DOOR, ACTION_SPAWN_EXTRAPERLO_DOOR_REAL</t>
@@ -14608,7 +14608,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="36" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="35">
@@ -25226,16 +25226,16 @@
         <v>0</v>
       </c>
       <c r="F94" s="44" t="s">
-        <v>705</v>
+        <v>479</v>
       </c>
       <c r="G94" s="39" t="s">
-        <v>479</v>
+        <v>627</v>
       </c>
       <c r="H94" s="44" t="s">
         <v>545</v>
       </c>
       <c r="I94" s="39" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="95">
@@ -25244,7 +25244,7 @@
         <v>29</v>
       </c>
       <c r="B95" s="45" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="C95" s="43" t="b">
         <v>0</v>
@@ -25259,7 +25259,7 @@
         <v>479</v>
       </c>
       <c r="G95" s="39" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="H95" s="44" t="s">
         <v>545</v>
@@ -31594,7 +31594,7 @@
         <v>727</v>
       </c>
       <c r="I229" s="48" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="J229" s="44" t="s">
         <v>728</v>
@@ -31669,7 +31669,7 @@
         <v>131</v>
       </c>
       <c r="B231" s="45" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C231" s="43" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Big changes on animation system
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7715" uniqueCount="2242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7728" uniqueCount="2255">
   <si>
     <t>NewItem</t>
   </si>
@@ -2435,7 +2435,7 @@
     <t>PHRASE_NONE</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_NONE</t>
+    <t>ANIMATION_TRIGGER_ZERO</t>
   </si>
   <si>
     <t>ANIMATION_NONE</t>
@@ -2972,7 +2972,7 @@
     <t>ACTION_ANIMATE_SILVANA_CLOSING_BOOK</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_TRANSITION_TWO</t>
+    <t>ANIMATION_TRIGGER_TWO</t>
   </si>
   <si>
     <t>ACTION_TALK_DIALOG_SILVANA_EXTRAPERLO</t>
@@ -2984,7 +2984,7 @@
     <t>ACTION_ANIMATE_SILVANA_OPENING_BOOK</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_TRANSITION_ONE</t>
+    <t>ANIMATION_TRIGGER_THREE</t>
   </si>
   <si>
     <t>ACTION_EVENT_SILVANA_REFUSED_MAINCHAR</t>
@@ -4871,7 +4871,7 @@
     <t>Text_Spanish</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_TALK</t>
+    <t>ANIMATION_TRIGGER_TALK_ONE</t>
   </si>
   <si>
     <t>That has no sense!</t>
@@ -4937,7 +4937,7 @@
     <t>PHRASE_DIALOG_REME_INTRO_2</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_STEADY</t>
+    <t>ANIMATION_TRIGGER_STEADY_ONE</t>
   </si>
   <si>
     <t>Be careful! It's just cleaned</t>
@@ -5864,9 +5864,6 @@
     <t>PHRASE_DIALOG_FIK_1_OPTION_1_3</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_THREE</t>
-  </si>
-  <si>
     <t>A ver chulo. Dime la frase para que te deje pasar</t>
   </si>
   <si>
@@ -5885,9 +5882,6 @@
     <t>PHRASE_DIALOG_FIK_1_OPTION_2_2</t>
   </si>
   <si>
-    <t>ANIMATION_TRIGGER_TWO</t>
-  </si>
-  <si>
     <t>...</t>
   </si>
   <si>
@@ -6380,301 +6374,346 @@
     <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_0_1</t>
   </si>
   <si>
+    <t>¿En serio vas a entrarme con esa mmm... basura de pregunta?</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_0_2</t>
+  </si>
+  <si>
+    <t>Te lo preguntaba en serio</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_0_3</t>
+  </si>
+  <si>
+    <t>Lamentaaable...</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_1_0</t>
+  </si>
+  <si>
+    <t>¿Tú conoces la fábrica de harina de las afueras?</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_1_1</t>
+  </si>
+  <si>
+    <t>Mira. No vayas por ahí. Los problemas que tengas con mi padre ¡Los hablas con mi padre!. Y como sigas me voy de aquí</t>
+  </si>
+  <si>
+    <t>¡Que tengas una buena noche!</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_INTRO_0</t>
+  </si>
+  <si>
+    <t>¿Os podéis cortar un poco de mirarme tý y el payaso ese?</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_INTRO_1</t>
+  </si>
+  <si>
+    <t>¡Ya sabes que el fin justifica los medios!</t>
+  </si>
+  <si>
+    <t>PHRASE_DIALOG_LAST</t>
+  </si>
+  <si>
+    <t>Last one</t>
+  </si>
+  <si>
+    <t>ROOM_ID</t>
+  </si>
+  <si>
+    <t>BackgroundSprite</t>
+  </si>
+  <si>
+    <t>BackgroundMusic</t>
+  </si>
+  <si>
+    <t>NeededBackgrounds_Sprites</t>
+  </si>
+  <si>
+    <t>NeededItems</t>
+  </si>
+  <si>
+    <t>NeededNames</t>
+  </si>
+  <si>
+    <t>NeededSounds</t>
+  </si>
+  <si>
+    <t>BackgroundActionConditions (6s)</t>
+  </si>
+  <si>
+    <t>OnEntryConditions</t>
+  </si>
+  <si>
+    <t>OnExitConditions</t>
+  </si>
+  <si>
+    <t>ROOM_NONE</t>
+  </si>
+  <si>
+    <t>HIVE1_ROOM_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_HIVE1_ROOM1, SPRITE_ITEM_DECO_BED_LAYER</t>
+  </si>
+  <si>
+    <t>ITEM_CARDS_PICKABLE, ITEM_HIVE1_CHEST, ITEM_HIVE1_WARDROBE, ITEM_HIVE1_WARDROBE_OPENED, ITEM_GENERIC_DOOR1, ITEM_HIVE1_PERFUME, ITEM_SOAP_PICKABLE, ITEM_HIVE1_BED</t>
+  </si>
+  <si>
+    <t>HIVE1_CORRIDOR_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_HIVE1_CORRIDOR1, BACKGROUND_HIVE1_CORRIDOR1_N</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_HIVE1_NPC_REME</t>
+  </si>
+  <si>
+    <t>HIVE1_HALL_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_HIVE1_HALL1, BACKGROUND_HIVE1_HALL1_N</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_GENERIC_DOOR2, ITEM_HIVE1_AD_BOARD, ITEM_HIVE1_EXIT_DOOR, ITEM_HIVE1_POOR_MAN_WC, ITEM_HIVE1_SHOELACE, ITEM_HIVE1_MAN_WC_CURED</t>
+  </si>
+  <si>
+    <t>HIVE1_WC_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_HIVE1_WC, BACKGROUND_HIVE1_WC_N</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_HIVE1_BASIN, ITEM_HIVE1_POOR_MAN_WC, ITEM_HIVE1_ROACH_HEAD, ITEM_HIVE1_PIPE</t>
+  </si>
+  <si>
+    <t>CITY1_STREET_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_STREET1, BACKGROUND_CITY1_STREET1_N</t>
+  </si>
+  <si>
+    <t>SOUND_AMBIENCE_CITY_DAY, SOUND_AMBIENCE_CITY_NIGHT</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_STREET1_STH_DOOR, ITEM_STREET1_CENTER_DOOR</t>
+  </si>
+  <si>
+    <t>CITY1_STREET_2</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_STREET2, BACKGROUND_CITY1_STREET2_N</t>
+  </si>
+  <si>
+    <t>ITEM_STREET2_PERIPH_DOOR, ITEM_PHARMACY_DOOR, ITEM_ELMANYO_DOOR</t>
+  </si>
+  <si>
+    <t>PHARMACY_1</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_PHARMACY_NPC_QUEUE, ITEM_PHARMACY_NPC_OWNER, ITEM_PHARMACY_INKWELL, ITEM_PHARMACY_INK</t>
+  </si>
+  <si>
+    <t>MANYO_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_MANYO, BACKGROUND_CITY1_MANYO_NIGHT</t>
+  </si>
+  <si>
+    <t>ITEM_CITY1_UMBRELLA, ITEM_GENERIC_DOOR1, ITEM_ELMANYO_OWNER, ITEM_STUFFED_DEER, ITEM_ELMANYO_OWNER_NIGHT, ITEM_ELMANYO_CROWD</t>
+  </si>
+  <si>
+    <t>MUSIC_MANYO, SOUND_AMBIENCE_MANYO_NIGHT</t>
+  </si>
+  <si>
+    <t>HIVE1_BACKALLEY</t>
+  </si>
+  <si>
+    <t>BACKGROUND_BACKALLEY, BACKGROUND_BACKALLEY_NIGHT</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_HIVE1_VALVE_BOX, ITEM_HIVE1_BACKALLEY_PIPE, ITEM_HIVE1_VALVE, ITEM_HIVE1_WATER_FLOWING</t>
+  </si>
+  <si>
+    <t>SOUND_AMBIENCE_CITY_DAY, SOUND_AMBIENCE_CITY_NIGHT, SOUND_AMBIENCE_WATER_FLOW</t>
+  </si>
+  <si>
+    <t>CITY1_SOUTH_STREET_1</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_SOUTH_STREET_1, BACKGROUND_CITY1_SOUTH_STREET_1_NIGHT</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_GENERIC_DOOR2</t>
+  </si>
+  <si>
+    <t>CITY1_SOUTH_STREET_2</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_SOUTH_STREET_2, BACKGROUND_CITY1_SOUTH_STREET_2_NIGHT</t>
+  </si>
+  <si>
+    <t>MUSIC_SOUTH_NEIGH, SOUND_AMBIENCE_CITY_NIGHT</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_NPC_FIK, ITEM_DOOR_EXTRAPERLO, ITEM_FOREGROUND_EXTRP_WALL, ITEM_DOOR_EXTRAPERLO_REAL, ITEM_NPC_GERMAN</t>
+  </si>
+  <si>
+    <t>MUSIC_SOUTH_NEIGH, SOUND_AMBIENCE_CITY_NIGHT, SOUND_AMBIENCE_OUTSIDE_PUB</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_EXTRAPERLO, SPRITE_EXTRAPERLO_BAR_FOREGROUND, SPRITE_EXTRAPERLO_COUPLE_TALKING</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_NPC_WAITER, ITEM_GENERIC_DOOR2, ITEM_NPC_UNKNOWN_WOMEN</t>
+  </si>
+  <si>
+    <t>MUSIC_EXTRAPERLO, SOUND_AMBIENCE_INSIDE_PUB</t>
+  </si>
+  <si>
+    <t>BACKGROUND_CITY1_EXTRAPERLO2, SPRITE_FIRE_DANCING, SPRITE_EXTRAPERLO_TABLE1_STEADY, SPRITE_EXTRAPERLO_TABLE2_STEADY</t>
+  </si>
+  <si>
+    <t>ITEM_GENERIC_DOOR1, ITEM_NPC_ARTURO_EXTRAPERLO, ITEM_NPC_CLOWN, ITEM_NPC_SILVANA_EXTRAPERLO</t>
+  </si>
+  <si>
+    <t>SOUND_AMBIENCE_INSIDE_PUB, MUSIC_EXTRAPERLO</t>
+  </si>
+  <si>
+    <t>ROOM_LAST</t>
+  </si>
+  <si>
+    <t>CHARACTER_TYPE_ID</t>
+  </si>
+  <si>
+    <t>CHARACTER_PARROT</t>
+  </si>
+  <si>
+    <t>CHARACTER_SNAKE</t>
+  </si>
+  <si>
+    <t>ANIMATION_ID</t>
+  </si>
+  <si>
+    <t>ITEM_USE_ANIMATION_NONE</t>
+  </si>
+  <si>
+    <t>ITEM_USE_ANIMATION_NORMAL</t>
+  </si>
+  <si>
+    <t>ITEM_USE_ANIMATION_TAKE</t>
+  </si>
+  <si>
+    <t>ITEM_USE_ANIMATION_CONFUSE</t>
+  </si>
+  <si>
+    <t>ITEM_USE_ANIMATION_STARE_SCREEN</t>
+  </si>
+  <si>
+    <t>ITEM_USE_ANIMATION_POUR</t>
+  </si>
+  <si>
+    <t>INTERACTION_ID</t>
+  </si>
+  <si>
+    <t>INTERACTION_MOVE</t>
+  </si>
+  <si>
+    <t>INTERACTION_COMBINE</t>
+  </si>
+  <si>
+    <t>ACTION_TYPE_ID</t>
+  </si>
+  <si>
+    <t>ACTION_TYPE_UNCLICKABLE</t>
+  </si>
+  <si>
+    <t>ACTION_TYPE_LOSE_ITEM</t>
+  </si>
+  <si>
+    <t>ACTION_TYPE_NOTIF</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_ID</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>No trigger</t>
+  </si>
+  <si>
+    <t>One shot triggers (auto return to auto steady)</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_FIVE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_SIX</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_SEVEN</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_EIGHT</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_ONE</t>
+  </si>
+  <si>
+    <t>Triggers which involve sub state machine then back to auto steady</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_THREE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_FOUR</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_FIVE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_SIX</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_SEVEN</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_CYCLE_EIGHT</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_STEADY_THREE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_STEADY_FOUR</t>
+  </si>
+  <si>
+    <t>Same as cycle but named as talk</t>
+  </si>
+  <si>
     <t>ANIMATION_TRIGGER_TALK_TWO</t>
   </si>
   <si>
-    <t>¿En serio vas a entrarme con esa mmm... basura de pregunta?</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_0_2</t>
-  </si>
-  <si>
-    <t>Te lo preguntaba en serio</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_0_3</t>
-  </si>
-  <si>
-    <t>Lamentaaable...</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_1_0</t>
-  </si>
-  <si>
-    <t>¿Tú conoces la fábrica de harina de las afueras?</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_OPTION_1_1</t>
-  </si>
-  <si>
-    <t>Mira. No vayas por ahí. Los problemas que tengas con mi padre ¡Los hablas con mi padre!. Y como sigas me voy de aquí</t>
-  </si>
-  <si>
-    <t>¡Que tengas una buena noche!</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_INTRO_0</t>
-  </si>
-  <si>
-    <t>¿Os podéis cortar un poco de mirarme tý y el payaso ese?</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_SILVANA_EXTRAPERLO_INTRO_1</t>
-  </si>
-  <si>
-    <t>¡Ya sabes que el fin justifica los medios!</t>
-  </si>
-  <si>
-    <t>PHRASE_DIALOG_LAST</t>
-  </si>
-  <si>
-    <t>Last one</t>
-  </si>
-  <si>
-    <t>ROOM_ID</t>
-  </si>
-  <si>
-    <t>BackgroundSprite</t>
-  </si>
-  <si>
-    <t>BackgroundMusic</t>
-  </si>
-  <si>
-    <t>NeededBackgrounds_Sprites</t>
-  </si>
-  <si>
-    <t>NeededItems</t>
-  </si>
-  <si>
-    <t>NeededNames</t>
-  </si>
-  <si>
-    <t>NeededSounds</t>
-  </si>
-  <si>
-    <t>BackgroundActionConditions (6s)</t>
-  </si>
-  <si>
-    <t>OnEntryConditions</t>
-  </si>
-  <si>
-    <t>OnExitConditions</t>
-  </si>
-  <si>
-    <t>ROOM_NONE</t>
-  </si>
-  <si>
-    <t>HIVE1_ROOM_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_HIVE1_ROOM1, SPRITE_ITEM_DECO_BED_LAYER</t>
-  </si>
-  <si>
-    <t>ITEM_CARDS_PICKABLE, ITEM_HIVE1_CHEST, ITEM_HIVE1_WARDROBE, ITEM_HIVE1_WARDROBE_OPENED, ITEM_GENERIC_DOOR1, ITEM_HIVE1_PERFUME, ITEM_SOAP_PICKABLE, ITEM_HIVE1_BED</t>
-  </si>
-  <si>
-    <t>HIVE1_CORRIDOR_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_HIVE1_CORRIDOR1, BACKGROUND_HIVE1_CORRIDOR1_N</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_HIVE1_NPC_REME</t>
-  </si>
-  <si>
-    <t>HIVE1_HALL_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_HIVE1_HALL1, BACKGROUND_HIVE1_HALL1_N</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_GENERIC_DOOR2, ITEM_HIVE1_AD_BOARD, ITEM_HIVE1_EXIT_DOOR, ITEM_HIVE1_POOR_MAN_WC, ITEM_HIVE1_SHOELACE, ITEM_HIVE1_MAN_WC_CURED</t>
-  </si>
-  <si>
-    <t>HIVE1_WC_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_HIVE1_WC, BACKGROUND_HIVE1_WC_N</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_HIVE1_BASIN, ITEM_HIVE1_POOR_MAN_WC, ITEM_HIVE1_ROACH_HEAD, ITEM_HIVE1_PIPE</t>
-  </si>
-  <si>
-    <t>CITY1_STREET_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_STREET1, BACKGROUND_CITY1_STREET1_N</t>
-  </si>
-  <si>
-    <t>SOUND_AMBIENCE_CITY_DAY, SOUND_AMBIENCE_CITY_NIGHT</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_STREET1_STH_DOOR, ITEM_STREET1_CENTER_DOOR</t>
-  </si>
-  <si>
-    <t>CITY1_STREET_2</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_STREET2, BACKGROUND_CITY1_STREET2_N</t>
-  </si>
-  <si>
-    <t>ITEM_STREET2_PERIPH_DOOR, ITEM_PHARMACY_DOOR, ITEM_ELMANYO_DOOR</t>
-  </si>
-  <si>
-    <t>PHARMACY_1</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_PHARMACY_NPC_QUEUE, ITEM_PHARMACY_NPC_OWNER, ITEM_PHARMACY_INKWELL, ITEM_PHARMACY_INK</t>
-  </si>
-  <si>
-    <t>MANYO_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_MANYO, BACKGROUND_CITY1_MANYO_NIGHT</t>
-  </si>
-  <si>
-    <t>ITEM_CITY1_UMBRELLA, ITEM_GENERIC_DOOR1, ITEM_ELMANYO_OWNER, ITEM_STUFFED_DEER, ITEM_ELMANYO_OWNER_NIGHT, ITEM_ELMANYO_CROWD</t>
-  </si>
-  <si>
-    <t>MUSIC_MANYO, SOUND_AMBIENCE_MANYO_NIGHT</t>
-  </si>
-  <si>
-    <t>HIVE1_BACKALLEY</t>
-  </si>
-  <si>
-    <t>BACKGROUND_BACKALLEY, BACKGROUND_BACKALLEY_NIGHT</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_HIVE1_VALVE_BOX, ITEM_HIVE1_BACKALLEY_PIPE, ITEM_HIVE1_VALVE, ITEM_HIVE1_WATER_FLOWING</t>
-  </si>
-  <si>
-    <t>SOUND_AMBIENCE_CITY_DAY, SOUND_AMBIENCE_CITY_NIGHT, SOUND_AMBIENCE_WATER_FLOW</t>
-  </si>
-  <si>
-    <t>CITY1_SOUTH_STREET_1</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_SOUTH_STREET_1, BACKGROUND_CITY1_SOUTH_STREET_1_NIGHT</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_GENERIC_DOOR2</t>
-  </si>
-  <si>
-    <t>CITY1_SOUTH_STREET_2</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_SOUTH_STREET_2, BACKGROUND_CITY1_SOUTH_STREET_2_NIGHT</t>
-  </si>
-  <si>
-    <t>MUSIC_SOUTH_NEIGH, SOUND_AMBIENCE_CITY_NIGHT</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_NPC_FIK, ITEM_DOOR_EXTRAPERLO, ITEM_FOREGROUND_EXTRP_WALL, ITEM_DOOR_EXTRAPERLO_REAL, ITEM_NPC_GERMAN</t>
-  </si>
-  <si>
-    <t>MUSIC_SOUTH_NEIGH, SOUND_AMBIENCE_CITY_NIGHT, SOUND_AMBIENCE_OUTSIDE_PUB</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_EXTRAPERLO, SPRITE_EXTRAPERLO_BAR_FOREGROUND, SPRITE_EXTRAPERLO_COUPLE_TALKING</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_NPC_WAITER, ITEM_GENERIC_DOOR2, ITEM_NPC_UNKNOWN_WOMEN</t>
-  </si>
-  <si>
-    <t>MUSIC_EXTRAPERLO, SOUND_AMBIENCE_INSIDE_PUB</t>
-  </si>
-  <si>
-    <t>BACKGROUND_CITY1_EXTRAPERLO2, SPRITE_FIRE_DANCING, SPRITE_EXTRAPERLO_TABLE1_STEADY, SPRITE_EXTRAPERLO_TABLE2_STEADY</t>
-  </si>
-  <si>
-    <t>ITEM_GENERIC_DOOR1, ITEM_NPC_ARTURO_EXTRAPERLO, ITEM_NPC_CLOWN, ITEM_NPC_SILVANA_EXTRAPERLO</t>
-  </si>
-  <si>
-    <t>SOUND_AMBIENCE_INSIDE_PUB, MUSIC_EXTRAPERLO</t>
-  </si>
-  <si>
-    <t>ROOM_LAST</t>
-  </si>
-  <si>
-    <t>CHARACTER_TYPE_ID</t>
-  </si>
-  <si>
-    <t>CHARACTER_PARROT</t>
-  </si>
-  <si>
-    <t>CHARACTER_SNAKE</t>
-  </si>
-  <si>
-    <t>ANIMATION_ID</t>
-  </si>
-  <si>
-    <t>ITEM_USE_ANIMATION_NONE</t>
-  </si>
-  <si>
-    <t>ITEM_USE_ANIMATION_NORMAL</t>
-  </si>
-  <si>
-    <t>ITEM_USE_ANIMATION_TAKE</t>
-  </si>
-  <si>
-    <t>ITEM_USE_ANIMATION_CONFUSE</t>
-  </si>
-  <si>
-    <t>ITEM_USE_ANIMATION_STARE_SCREEN</t>
-  </si>
-  <si>
-    <t>ITEM_USE_ANIMATION_POUR</t>
-  </si>
-  <si>
-    <t>INTERACTION_ID</t>
-  </si>
-  <si>
-    <t>INTERACTION_MOVE</t>
-  </si>
-  <si>
-    <t>INTERACTION_COMBINE</t>
-  </si>
-  <si>
-    <t>ACTION_TYPE_ID</t>
-  </si>
-  <si>
-    <t>ACTION_TYPE_UNCLICKABLE</t>
-  </si>
-  <si>
-    <t>ACTION_TYPE_LOSE_ITEM</t>
-  </si>
-  <si>
-    <t>ACTION_TYPE_NOTIF</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_ID</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_FIVE</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_SIX</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_SEVEN</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_EIGHT</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_CYCLE_ONE</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_CYCLE_THREE</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_CYCLE_FOUR</t>
+    <t>ANIMATION_TRIGGER_TALK_THREE</t>
+  </si>
+  <si>
+    <t>ANIMATION_TRIGGER_TALK_FOUR</t>
   </si>
   <si>
     <t>ANIMATION_TRIGGER_AUTO_STEADY</t>
   </si>
   <si>
+    <t>Special trigger which takes las steady trigger taken</t>
+  </si>
+  <si>
     <t>ANIMATION_TRIGGER_WALK_FRONT</t>
+  </si>
+  <si>
+    <t>Character walks</t>
   </si>
   <si>
     <t>ANIMATION_TRIGGER_WALK_BACK</t>
@@ -8276,17 +8315,18 @@
 </file>
 
 <file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A45:B70" displayName="Table_Animation_Trigger" name="Table_Animation_Trigger" id="24">
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A45:C76" displayName="Table_Animation_Trigger" name="Table_Animation_Trigger" id="24">
+  <tableColumns count="3">
     <tableColumn name="N" id="1"/>
     <tableColumn name="ANIMATION_TRIGGER_ID" id="2"/>
+    <tableColumn name="Comment" id="3"/>
   </tableColumns>
   <tableStyleInfo name="TYPES-style 5" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A72:B77" displayName="Table_Item_Family_Type" name="Table_Item_Family_Type" id="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A78:B83" displayName="Table_Item_Family_Type" name="Table_Item_Family_Type" id="25">
   <tableColumns count="2">
     <tableColumn name="N" id="1"/>
     <tableColumn name="ITEM_FAMILY_TYPE_ID" id="2"/>
@@ -8296,7 +8336,7 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A79:B82" displayName="Table_Moment_Day" name="Table_Moment_Day" id="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A85:B88" displayName="Table_Moment_Day" name="Table_Moment_Day" id="26">
   <tableColumns count="2">
     <tableColumn name="N" id="1"/>
     <tableColumn name="MOMENT_TYPE_ID" id="2"/>
@@ -13710,7 +13750,7 @@
         <v>1098</v>
       </c>
       <c r="E132" s="45" t="s">
-        <v>1920</v>
+        <v>960</v>
       </c>
       <c r="F132" s="39" t="s">
         <v>1589</v>
@@ -13719,10 +13759,10 @@
         <v>777</v>
       </c>
       <c r="H132" s="38" t="s">
-        <v>1921</v>
+        <v>1920</v>
       </c>
       <c r="I132" s="38" t="s">
-        <v>1921</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="133">
@@ -13731,7 +13771,7 @@
         <v>131</v>
       </c>
       <c r="B133" s="37" t="s">
-        <v>1922</v>
+        <v>1921</v>
       </c>
       <c r="C133" s="37">
         <v>0.0</v>
@@ -13749,10 +13789,10 @@
         <v>777</v>
       </c>
       <c r="H133" s="38" t="s">
-        <v>1923</v>
+        <v>1922</v>
       </c>
       <c r="I133" s="38" t="s">
-        <v>1923</v>
+        <v>1922</v>
       </c>
     </row>
     <row r="134">
@@ -13761,7 +13801,7 @@
         <v>132</v>
       </c>
       <c r="B134" s="37" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="C134" s="37">
         <v>1.0</v>
@@ -13779,10 +13819,10 @@
         <v>777</v>
       </c>
       <c r="H134" s="38" t="s">
-        <v>1925</v>
+        <v>1924</v>
       </c>
       <c r="I134" s="38" t="s">
-        <v>1925</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="135">
@@ -13791,7 +13831,7 @@
         <v>133</v>
       </c>
       <c r="B135" s="37" t="s">
-        <v>1926</v>
+        <v>1925</v>
       </c>
       <c r="C135" s="37">
         <v>0.0</v>
@@ -13800,7 +13840,7 @@
         <v>1066</v>
       </c>
       <c r="E135" s="45" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
       <c r="F135" s="39" t="s">
         <v>1611</v>
@@ -13809,10 +13849,10 @@
         <v>777</v>
       </c>
       <c r="H135" s="38" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
       <c r="I135" s="38" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="136">
@@ -13839,10 +13879,10 @@
         <v>777</v>
       </c>
       <c r="H136" s="38" t="s">
-        <v>1929</v>
+        <v>1927</v>
       </c>
       <c r="I136" s="38" t="s">
-        <v>1930</v>
+        <v>1928</v>
       </c>
     </row>
     <row r="137">
@@ -13851,7 +13891,7 @@
         <v>135</v>
       </c>
       <c r="B137" s="37" t="s">
-        <v>1931</v>
+        <v>1929</v>
       </c>
       <c r="C137" s="37">
         <v>1.0</v>
@@ -13869,10 +13909,10 @@
         <v>777</v>
       </c>
       <c r="H137" s="38" t="s">
-        <v>1932</v>
+        <v>1930</v>
       </c>
       <c r="I137" s="38" t="s">
-        <v>1932</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="138">
@@ -13881,7 +13921,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="37" t="s">
-        <v>1933</v>
+        <v>1931</v>
       </c>
       <c r="C138" s="37">
         <v>1.0</v>
@@ -13899,10 +13939,10 @@
         <v>777</v>
       </c>
       <c r="H138" s="38" t="s">
-        <v>1934</v>
+        <v>1932</v>
       </c>
       <c r="I138" s="38" t="s">
-        <v>1934</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="139">
@@ -13911,7 +13951,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="37" t="s">
-        <v>1935</v>
+        <v>1933</v>
       </c>
       <c r="C139" s="37">
         <v>0.0</v>
@@ -13920,7 +13960,7 @@
         <v>1106</v>
       </c>
       <c r="E139" s="45" t="s">
-        <v>1936</v>
+        <v>1934</v>
       </c>
       <c r="F139" s="39" t="s">
         <v>1611</v>
@@ -13929,10 +13969,10 @@
         <v>777</v>
       </c>
       <c r="H139" s="38" t="s">
-        <v>1937</v>
+        <v>1935</v>
       </c>
       <c r="I139" s="38" t="s">
-        <v>1937</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="140">
@@ -13941,7 +13981,7 @@
         <v>138</v>
       </c>
       <c r="B140" s="37" t="s">
-        <v>1938</v>
+        <v>1936</v>
       </c>
       <c r="C140" s="37">
         <v>1.0</v>
@@ -13950,7 +13990,7 @@
         <v>1108</v>
       </c>
       <c r="E140" s="45" t="s">
-        <v>1920</v>
+        <v>960</v>
       </c>
       <c r="F140" s="39" t="s">
         <v>1589</v>
@@ -13959,10 +13999,10 @@
         <v>777</v>
       </c>
       <c r="H140" s="38" t="s">
-        <v>1939</v>
+        <v>1937</v>
       </c>
       <c r="I140" s="38" t="s">
-        <v>1939</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="141">
@@ -13971,7 +14011,7 @@
         <v>139</v>
       </c>
       <c r="B141" s="37" t="s">
-        <v>1940</v>
+        <v>1938</v>
       </c>
       <c r="C141" s="37">
         <v>0.0</v>
@@ -13980,7 +14020,7 @@
         <v>1110</v>
       </c>
       <c r="E141" s="45" t="s">
-        <v>1936</v>
+        <v>1934</v>
       </c>
       <c r="F141" s="39" t="s">
         <v>1611</v>
@@ -13989,10 +14029,10 @@
         <v>777</v>
       </c>
       <c r="H141" s="38" t="s">
-        <v>1941</v>
+        <v>1939</v>
       </c>
       <c r="I141" s="38" t="s">
-        <v>1941</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="142">
@@ -14001,7 +14041,7 @@
         <v>140</v>
       </c>
       <c r="B142" s="37" t="s">
-        <v>1942</v>
+        <v>1940</v>
       </c>
       <c r="C142" s="37">
         <v>1.0</v>
@@ -14010,7 +14050,7 @@
         <v>1112</v>
       </c>
       <c r="E142" s="45" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
       <c r="F142" s="39" t="s">
         <v>1589</v>
@@ -14019,10 +14059,10 @@
         <v>777</v>
       </c>
       <c r="H142" s="38" t="s">
-        <v>1943</v>
+        <v>1941</v>
       </c>
       <c r="I142" s="38" t="s">
-        <v>1943</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="143">
@@ -14031,7 +14071,7 @@
         <v>141</v>
       </c>
       <c r="B143" s="37" t="s">
-        <v>1944</v>
+        <v>1942</v>
       </c>
       <c r="C143" s="37">
         <v>0.0</v>
@@ -14040,7 +14080,7 @@
         <v>1114</v>
       </c>
       <c r="E143" s="45" t="s">
-        <v>1936</v>
+        <v>1934</v>
       </c>
       <c r="F143" s="39" t="s">
         <v>1611</v>
@@ -14049,10 +14089,10 @@
         <v>777</v>
       </c>
       <c r="H143" s="38" t="s">
-        <v>1945</v>
+        <v>1943</v>
       </c>
       <c r="I143" s="38" t="s">
-        <v>1945</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="144">
@@ -14061,7 +14101,7 @@
         <v>142</v>
       </c>
       <c r="B144" s="37" t="s">
-        <v>1946</v>
+        <v>1944</v>
       </c>
       <c r="C144" s="37">
         <v>1.0</v>
@@ -14070,7 +14110,7 @@
         <v>1116</v>
       </c>
       <c r="E144" s="45" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
       <c r="F144" s="39" t="s">
         <v>1589</v>
@@ -14079,10 +14119,10 @@
         <v>777</v>
       </c>
       <c r="H144" s="38" t="s">
-        <v>1947</v>
+        <v>1945</v>
       </c>
       <c r="I144" s="38" t="s">
-        <v>1947</v>
+        <v>1945</v>
       </c>
     </row>
     <row r="145">
@@ -14091,7 +14131,7 @@
         <v>143</v>
       </c>
       <c r="B145" s="37" t="s">
-        <v>1948</v>
+        <v>1946</v>
       </c>
       <c r="C145" s="37">
         <v>0.0</v>
@@ -14109,10 +14149,10 @@
         <v>777</v>
       </c>
       <c r="H145" s="38" t="s">
-        <v>1949</v>
+        <v>1947</v>
       </c>
       <c r="I145" s="38" t="s">
-        <v>1949</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="146">
@@ -14121,7 +14161,7 @@
         <v>144</v>
       </c>
       <c r="B146" s="37" t="s">
-        <v>1950</v>
+        <v>1948</v>
       </c>
       <c r="C146" s="37">
         <v>1.0</v>
@@ -14139,10 +14179,10 @@
         <v>777</v>
       </c>
       <c r="H146" s="38" t="s">
-        <v>1951</v>
+        <v>1949</v>
       </c>
       <c r="I146" s="38" t="s">
-        <v>1951</v>
+        <v>1949</v>
       </c>
     </row>
     <row r="147">
@@ -14169,10 +14209,10 @@
         <v>777</v>
       </c>
       <c r="H147" s="38" t="s">
-        <v>1952</v>
+        <v>1950</v>
       </c>
       <c r="I147" s="38" t="s">
-        <v>1952</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="148">
@@ -14181,7 +14221,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="37" t="s">
-        <v>1953</v>
+        <v>1951</v>
       </c>
       <c r="C148" s="37">
         <v>0.0</v>
@@ -14199,10 +14239,10 @@
         <v>777</v>
       </c>
       <c r="H148" s="38" t="s">
-        <v>1954</v>
+        <v>1952</v>
       </c>
       <c r="I148" s="38" t="s">
-        <v>1954</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="149">
@@ -14211,7 +14251,7 @@
         <v>147</v>
       </c>
       <c r="B149" s="37" t="s">
-        <v>1955</v>
+        <v>1953</v>
       </c>
       <c r="C149" s="37">
         <v>1.0</v>
@@ -14229,10 +14269,10 @@
         <v>777</v>
       </c>
       <c r="H149" s="38" t="s">
-        <v>1956</v>
+        <v>1954</v>
       </c>
       <c r="I149" s="38" t="s">
-        <v>1956</v>
+        <v>1954</v>
       </c>
     </row>
     <row r="150">
@@ -14241,7 +14281,7 @@
         <v>148</v>
       </c>
       <c r="B150" s="37" t="s">
-        <v>1957</v>
+        <v>1955</v>
       </c>
       <c r="C150" s="37">
         <v>0.0</v>
@@ -14259,10 +14299,10 @@
         <v>777</v>
       </c>
       <c r="H150" s="38" t="s">
-        <v>1958</v>
+        <v>1956</v>
       </c>
       <c r="I150" s="38" t="s">
-        <v>1958</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="151">
@@ -14271,7 +14311,7 @@
         <v>149</v>
       </c>
       <c r="B151" s="37" t="s">
-        <v>1959</v>
+        <v>1957</v>
       </c>
       <c r="C151" s="37">
         <v>1.0</v>
@@ -14289,10 +14329,10 @@
         <v>777</v>
       </c>
       <c r="H151" s="38" t="s">
-        <v>1960</v>
+        <v>1958</v>
       </c>
       <c r="I151" s="38" t="s">
-        <v>1960</v>
+        <v>1958</v>
       </c>
     </row>
     <row r="152">
@@ -14301,7 +14341,7 @@
         <v>150</v>
       </c>
       <c r="B152" s="37" t="s">
-        <v>1961</v>
+        <v>1959</v>
       </c>
       <c r="C152" s="37">
         <v>0.0</v>
@@ -14319,10 +14359,10 @@
         <v>777</v>
       </c>
       <c r="H152" s="38" t="s">
-        <v>1962</v>
+        <v>1960</v>
       </c>
       <c r="I152" s="38" t="s">
-        <v>1962</v>
+        <v>1960</v>
       </c>
     </row>
     <row r="153">
@@ -14331,7 +14371,7 @@
         <v>151</v>
       </c>
       <c r="B153" s="37" t="s">
-        <v>1963</v>
+        <v>1961</v>
       </c>
       <c r="C153" s="37">
         <v>1.0</v>
@@ -14349,10 +14389,10 @@
         <v>777</v>
       </c>
       <c r="H153" s="38" t="s">
-        <v>1964</v>
+        <v>1962</v>
       </c>
       <c r="I153" s="38" t="s">
-        <v>1964</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="154">
@@ -14361,7 +14401,7 @@
         <v>152</v>
       </c>
       <c r="B154" s="37" t="s">
-        <v>1965</v>
+        <v>1963</v>
       </c>
       <c r="C154" s="37">
         <v>0.0</v>
@@ -14370,7 +14410,7 @@
         <v>1066</v>
       </c>
       <c r="E154" s="45" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
       <c r="F154" s="39" t="s">
         <v>1611</v>
@@ -14379,10 +14419,10 @@
         <v>777</v>
       </c>
       <c r="H154" s="38" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
       <c r="I154" s="38" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="155">
@@ -14409,10 +14449,10 @@
         <v>777</v>
       </c>
       <c r="H155" s="38" t="s">
-        <v>1966</v>
+        <v>1964</v>
       </c>
       <c r="I155" s="38" t="s">
-        <v>1966</v>
+        <v>1964</v>
       </c>
     </row>
     <row r="156">
@@ -14421,7 +14461,7 @@
         <v>154</v>
       </c>
       <c r="B156" s="37" t="s">
-        <v>1967</v>
+        <v>1965</v>
       </c>
       <c r="C156" s="37">
         <v>1.0</v>
@@ -14439,10 +14479,10 @@
         <v>777</v>
       </c>
       <c r="H156" s="38" t="s">
-        <v>1968</v>
+        <v>1966</v>
       </c>
       <c r="I156" s="38" t="s">
-        <v>1968</v>
+        <v>1966</v>
       </c>
     </row>
     <row r="157">
@@ -14451,7 +14491,7 @@
         <v>155</v>
       </c>
       <c r="B157" s="37" t="s">
-        <v>1969</v>
+        <v>1967</v>
       </c>
       <c r="C157" s="37">
         <v>0.0</v>
@@ -14469,10 +14509,10 @@
         <v>777</v>
       </c>
       <c r="H157" s="38" t="s">
-        <v>1970</v>
+        <v>1968</v>
       </c>
       <c r="I157" s="38" t="s">
-        <v>1970</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="158">
@@ -14481,7 +14521,7 @@
         <v>156</v>
       </c>
       <c r="B158" s="37" t="s">
-        <v>1971</v>
+        <v>1969</v>
       </c>
       <c r="C158" s="37">
         <v>1.0</v>
@@ -14499,10 +14539,10 @@
         <v>777</v>
       </c>
       <c r="H158" s="38" t="s">
-        <v>1972</v>
+        <v>1970</v>
       </c>
       <c r="I158" s="38" t="s">
-        <v>1972</v>
+        <v>1970</v>
       </c>
     </row>
     <row r="159">
@@ -14511,7 +14551,7 @@
         <v>157</v>
       </c>
       <c r="B159" s="37" t="s">
-        <v>1973</v>
+        <v>1971</v>
       </c>
       <c r="C159" s="37">
         <v>0.0</v>
@@ -14523,16 +14563,16 @@
         <v>1589</v>
       </c>
       <c r="F159" s="39" t="s">
-        <v>1974</v>
+        <v>1972</v>
       </c>
       <c r="G159" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H159" s="38" t="s">
-        <v>1975</v>
+        <v>1973</v>
       </c>
       <c r="I159" s="38" t="s">
-        <v>1975</v>
+        <v>1973</v>
       </c>
     </row>
     <row r="160">
@@ -14541,7 +14581,7 @@
         <v>158</v>
       </c>
       <c r="B160" s="37" t="s">
-        <v>1976</v>
+        <v>1974</v>
       </c>
       <c r="C160" s="37">
         <v>0.0</v>
@@ -14559,10 +14599,10 @@
         <v>777</v>
       </c>
       <c r="H160" s="38" t="s">
-        <v>1977</v>
+        <v>1975</v>
       </c>
       <c r="I160" s="38" t="s">
-        <v>1977</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="161">
@@ -14571,7 +14611,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="37" t="s">
-        <v>1978</v>
+        <v>1976</v>
       </c>
       <c r="C161" s="37">
         <v>1.0</v>
@@ -14589,10 +14629,10 @@
         <v>777</v>
       </c>
       <c r="H161" s="38" t="s">
-        <v>1979</v>
+        <v>1977</v>
       </c>
       <c r="I161" s="38" t="s">
-        <v>1979</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="162">
@@ -14601,7 +14641,7 @@
         <v>160</v>
       </c>
       <c r="B162" s="37" t="s">
-        <v>1980</v>
+        <v>1978</v>
       </c>
       <c r="C162" s="37">
         <v>0.0</v>
@@ -14613,16 +14653,16 @@
         <v>1589</v>
       </c>
       <c r="F162" s="39" t="s">
-        <v>1974</v>
+        <v>1972</v>
       </c>
       <c r="G162" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H162" s="38" t="s">
-        <v>1981</v>
+        <v>1979</v>
       </c>
       <c r="I162" s="38" t="s">
-        <v>1981</v>
+        <v>1979</v>
       </c>
     </row>
     <row r="163">
@@ -14631,7 +14671,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="37" t="s">
-        <v>1982</v>
+        <v>1980</v>
       </c>
       <c r="C163" s="37">
         <v>0.0</v>
@@ -14649,10 +14689,10 @@
         <v>777</v>
       </c>
       <c r="H163" s="38" t="s">
-        <v>1983</v>
+        <v>1981</v>
       </c>
       <c r="I163" s="38" t="s">
-        <v>1983</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="164">
@@ -14661,7 +14701,7 @@
         <v>162</v>
       </c>
       <c r="B164" s="37" t="s">
-        <v>1984</v>
+        <v>1982</v>
       </c>
       <c r="C164" s="37">
         <v>1.0</v>
@@ -14673,16 +14713,16 @@
         <v>1611</v>
       </c>
       <c r="F164" s="39" t="s">
-        <v>1974</v>
+        <v>1972</v>
       </c>
       <c r="G164" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H164" s="38" t="s">
-        <v>1985</v>
+        <v>1983</v>
       </c>
       <c r="I164" s="38" t="s">
-        <v>1985</v>
+        <v>1983</v>
       </c>
     </row>
     <row r="165">
@@ -14691,7 +14731,7 @@
         <v>163</v>
       </c>
       <c r="B165" s="37" t="s">
-        <v>1986</v>
+        <v>1984</v>
       </c>
       <c r="C165" s="37">
         <v>0.0</v>
@@ -14700,19 +14740,19 @@
         <v>1066</v>
       </c>
       <c r="E165" s="45" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
       <c r="F165" s="39" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
       <c r="G165" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H165" s="38" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
       <c r="I165" s="38" t="s">
-        <v>1928</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="166">
@@ -14739,10 +14779,10 @@
         <v>777</v>
       </c>
       <c r="H166" s="38" t="s">
-        <v>1987</v>
+        <v>1985</v>
       </c>
       <c r="I166" s="38" t="s">
-        <v>1987</v>
+        <v>1985</v>
       </c>
     </row>
     <row r="167">
@@ -14781,7 +14821,7 @@
         <v>166</v>
       </c>
       <c r="B168" s="37" t="s">
-        <v>1988</v>
+        <v>1986</v>
       </c>
       <c r="C168" s="37">
         <v>0.0</v>
@@ -14799,10 +14839,10 @@
         <v>777</v>
       </c>
       <c r="H168" s="38" t="s">
-        <v>1989</v>
+        <v>1987</v>
       </c>
       <c r="I168" s="38" t="s">
-        <v>1989</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="169">
@@ -14811,7 +14851,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="37" t="s">
-        <v>1990</v>
+        <v>1988</v>
       </c>
       <c r="C169" s="37">
         <v>1.0</v>
@@ -14829,10 +14869,10 @@
         <v>777</v>
       </c>
       <c r="H169" s="38" t="s">
-        <v>1991</v>
+        <v>1989</v>
       </c>
       <c r="I169" s="38" t="s">
-        <v>1991</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="170">
@@ -14841,7 +14881,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="37" t="s">
-        <v>1992</v>
+        <v>1990</v>
       </c>
       <c r="C170" s="37">
         <v>0.0</v>
@@ -14859,10 +14899,10 @@
         <v>777</v>
       </c>
       <c r="H170" s="38" t="s">
-        <v>1993</v>
+        <v>1991</v>
       </c>
       <c r="I170" s="38" t="s">
-        <v>1993</v>
+        <v>1991</v>
       </c>
     </row>
     <row r="171">
@@ -14871,7 +14911,7 @@
         <v>169</v>
       </c>
       <c r="B171" s="37" t="s">
-        <v>1994</v>
+        <v>1992</v>
       </c>
       <c r="C171" s="37">
         <v>1.0</v>
@@ -14889,10 +14929,10 @@
         <v>777</v>
       </c>
       <c r="H171" s="38" t="s">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="I171" s="38" t="s">
-        <v>1995</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="172">
@@ -14901,7 +14941,7 @@
         <v>170</v>
       </c>
       <c r="B172" s="37" t="s">
-        <v>1996</v>
+        <v>1994</v>
       </c>
       <c r="C172" s="37">
         <v>0.0</v>
@@ -14919,10 +14959,10 @@
         <v>777</v>
       </c>
       <c r="H172" s="38" t="s">
-        <v>1997</v>
+        <v>1995</v>
       </c>
       <c r="I172" s="38" t="s">
-        <v>1997</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="173">
@@ -14931,7 +14971,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="37" t="s">
-        <v>1998</v>
+        <v>1996</v>
       </c>
       <c r="C173" s="37">
         <v>1.0</v>
@@ -14949,10 +14989,10 @@
         <v>777</v>
       </c>
       <c r="H173" s="38" t="s">
-        <v>1999</v>
+        <v>1997</v>
       </c>
       <c r="I173" s="38" t="s">
-        <v>1999</v>
+        <v>1997</v>
       </c>
     </row>
     <row r="174">
@@ -14961,7 +15001,7 @@
         <v>172</v>
       </c>
       <c r="B174" s="37" t="s">
-        <v>2000</v>
+        <v>1998</v>
       </c>
       <c r="C174" s="37">
         <v>0.0</v>
@@ -14979,10 +15019,10 @@
         <v>777</v>
       </c>
       <c r="H174" s="38" t="s">
-        <v>2001</v>
+        <v>1999</v>
       </c>
       <c r="I174" s="38" t="s">
-        <v>2001</v>
+        <v>1999</v>
       </c>
     </row>
     <row r="175">
@@ -14991,7 +15031,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="37" t="s">
-        <v>2002</v>
+        <v>2000</v>
       </c>
       <c r="C175" s="37">
         <v>1.0</v>
@@ -15009,10 +15049,10 @@
         <v>777</v>
       </c>
       <c r="H175" s="38" t="s">
-        <v>2003</v>
+        <v>2001</v>
       </c>
       <c r="I175" s="38" t="s">
-        <v>2003</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="176">
@@ -15021,7 +15061,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="37" t="s">
-        <v>2004</v>
+        <v>2002</v>
       </c>
       <c r="C176" s="37">
         <v>0.0</v>
@@ -15039,10 +15079,10 @@
         <v>777</v>
       </c>
       <c r="H176" s="38" t="s">
-        <v>2005</v>
+        <v>2003</v>
       </c>
       <c r="I176" s="38" t="s">
-        <v>2005</v>
+        <v>2003</v>
       </c>
     </row>
     <row r="177">
@@ -15051,7 +15091,7 @@
         <v>175</v>
       </c>
       <c r="B177" s="37" t="s">
-        <v>2006</v>
+        <v>2004</v>
       </c>
       <c r="C177" s="37">
         <v>0.0</v>
@@ -15069,10 +15109,10 @@
         <v>777</v>
       </c>
       <c r="H177" s="38" t="s">
-        <v>2007</v>
+        <v>2005</v>
       </c>
       <c r="I177" s="38" t="s">
-        <v>2007</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="178">
@@ -15081,7 +15121,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="37" t="s">
-        <v>2008</v>
+        <v>2006</v>
       </c>
       <c r="C178" s="37">
         <v>1.0</v>
@@ -15099,10 +15139,10 @@
         <v>777</v>
       </c>
       <c r="H178" s="38" t="s">
-        <v>2009</v>
+        <v>2007</v>
       </c>
       <c r="I178" s="38" t="s">
-        <v>2009</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="179">
@@ -15111,7 +15151,7 @@
         <v>177</v>
       </c>
       <c r="B179" s="37" t="s">
-        <v>2010</v>
+        <v>2008</v>
       </c>
       <c r="C179" s="37">
         <v>1.0</v>
@@ -15129,10 +15169,10 @@
         <v>777</v>
       </c>
       <c r="H179" s="38" t="s">
-        <v>2011</v>
+        <v>2009</v>
       </c>
       <c r="I179" s="38" t="s">
-        <v>2011</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="180">
@@ -15141,7 +15181,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="37" t="s">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="C180" s="37">
         <v>0.0</v>
@@ -15159,10 +15199,10 @@
         <v>777</v>
       </c>
       <c r="H180" s="38" t="s">
-        <v>2013</v>
+        <v>2011</v>
       </c>
       <c r="I180" s="38" t="s">
-        <v>2013</v>
+        <v>2011</v>
       </c>
     </row>
     <row r="181">
@@ -15171,7 +15211,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="37" t="s">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="C181" s="37">
         <v>1.0</v>
@@ -15189,10 +15229,10 @@
         <v>777</v>
       </c>
       <c r="H181" s="38" t="s">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="I181" s="38" t="s">
-        <v>2015</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="182">
@@ -15201,7 +15241,7 @@
         <v>180</v>
       </c>
       <c r="B182" s="37" t="s">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="C182" s="37">
         <v>0.0</v>
@@ -15219,10 +15259,10 @@
         <v>777</v>
       </c>
       <c r="H182" s="38" t="s">
-        <v>2017</v>
+        <v>2015</v>
       </c>
       <c r="I182" s="38" t="s">
-        <v>2017</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="183">
@@ -15231,7 +15271,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="37" t="s">
-        <v>2018</v>
+        <v>2016</v>
       </c>
       <c r="C183" s="37">
         <v>1.0</v>
@@ -15249,10 +15289,10 @@
         <v>777</v>
       </c>
       <c r="H183" s="38" t="s">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="I183" s="38" t="s">
-        <v>2019</v>
+        <v>2017</v>
       </c>
     </row>
     <row r="184">
@@ -15261,7 +15301,7 @@
         <v>182</v>
       </c>
       <c r="B184" s="37" t="s">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="C184" s="37">
         <v>0.0</v>
@@ -15279,10 +15319,10 @@
         <v>777</v>
       </c>
       <c r="H184" s="38" t="s">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="I184" s="38" t="s">
-        <v>2021</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="185">
@@ -15309,10 +15349,10 @@
         <v>777</v>
       </c>
       <c r="H185" s="38" t="s">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="I185" s="38" t="s">
-        <v>2022</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="186">
@@ -15321,7 +15361,7 @@
         <v>184</v>
       </c>
       <c r="B186" s="37" t="s">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C186" s="37">
         <v>0.0</v>
@@ -15339,10 +15379,10 @@
         <v>777</v>
       </c>
       <c r="H186" s="38" t="s">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="I186" s="38" t="s">
-        <v>2024</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="187">
@@ -15351,7 +15391,7 @@
         <v>185</v>
       </c>
       <c r="B187" s="37" t="s">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="C187" s="37">
         <v>0.0</v>
@@ -15369,10 +15409,10 @@
         <v>777</v>
       </c>
       <c r="H187" s="38" t="s">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="I187" s="38" t="s">
-        <v>2026</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="188">
@@ -15381,7 +15421,7 @@
         <v>186</v>
       </c>
       <c r="B188" s="37" t="s">
-        <v>2027</v>
+        <v>2025</v>
       </c>
       <c r="C188" s="37">
         <v>0.0</v>
@@ -15399,10 +15439,10 @@
         <v>777</v>
       </c>
       <c r="H188" s="38" t="s">
-        <v>2028</v>
+        <v>2026</v>
       </c>
       <c r="I188" s="38" t="s">
-        <v>2028</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="189">
@@ -15411,7 +15451,7 @@
         <v>187</v>
       </c>
       <c r="B189" s="37" t="s">
-        <v>2029</v>
+        <v>2027</v>
       </c>
       <c r="C189" s="37">
         <v>0.0</v>
@@ -15429,10 +15469,10 @@
         <v>777</v>
       </c>
       <c r="H189" s="38" t="s">
-        <v>2030</v>
+        <v>2028</v>
       </c>
       <c r="I189" s="38" t="s">
-        <v>2030</v>
+        <v>2028</v>
       </c>
     </row>
     <row r="190">
@@ -15441,7 +15481,7 @@
         <v>188</v>
       </c>
       <c r="B190" s="37" t="s">
-        <v>2031</v>
+        <v>2029</v>
       </c>
       <c r="C190" s="37">
         <v>0.0</v>
@@ -15459,10 +15499,10 @@
         <v>777</v>
       </c>
       <c r="H190" s="38" t="s">
-        <v>2032</v>
+        <v>2030</v>
       </c>
       <c r="I190" s="38" t="s">
-        <v>2032</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="191">
@@ -15471,7 +15511,7 @@
         <v>189</v>
       </c>
       <c r="B191" s="37" t="s">
-        <v>2033</v>
+        <v>2031</v>
       </c>
       <c r="C191" s="37">
         <v>0.0</v>
@@ -15489,10 +15529,10 @@
         <v>777</v>
       </c>
       <c r="H191" s="38" t="s">
-        <v>2034</v>
+        <v>2032</v>
       </c>
       <c r="I191" s="38" t="s">
-        <v>2034</v>
+        <v>2032</v>
       </c>
     </row>
     <row r="192">
@@ -15501,7 +15541,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="37" t="s">
-        <v>2035</v>
+        <v>2033</v>
       </c>
       <c r="C192" s="37">
         <v>0.0</v>
@@ -15519,10 +15559,10 @@
         <v>777</v>
       </c>
       <c r="H192" s="38" t="s">
-        <v>2036</v>
+        <v>2034</v>
       </c>
       <c r="I192" s="38" t="s">
-        <v>2036</v>
+        <v>2034</v>
       </c>
     </row>
     <row r="193">
@@ -15531,7 +15571,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="37" t="s">
-        <v>2037</v>
+        <v>2035</v>
       </c>
       <c r="C193" s="37">
         <v>0.0</v>
@@ -15549,10 +15589,10 @@
         <v>777</v>
       </c>
       <c r="H193" s="38" t="s">
-        <v>2038</v>
+        <v>2036</v>
       </c>
       <c r="I193" s="38" t="s">
-        <v>2038</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="194">
@@ -15561,7 +15601,7 @@
         <v>192</v>
       </c>
       <c r="B194" s="37" t="s">
-        <v>2039</v>
+        <v>2037</v>
       </c>
       <c r="C194" s="37">
         <v>0.0</v>
@@ -15579,10 +15619,10 @@
         <v>777</v>
       </c>
       <c r="H194" s="38" t="s">
-        <v>2040</v>
+        <v>2038</v>
       </c>
       <c r="I194" s="38" t="s">
-        <v>2040</v>
+        <v>2038</v>
       </c>
     </row>
     <row r="195">
@@ -15591,7 +15631,7 @@
         <v>193</v>
       </c>
       <c r="B195" s="37" t="s">
-        <v>2041</v>
+        <v>2039</v>
       </c>
       <c r="C195" s="37">
         <v>0.0</v>
@@ -15609,10 +15649,10 @@
         <v>777</v>
       </c>
       <c r="H195" s="38" t="s">
-        <v>2042</v>
+        <v>2040</v>
       </c>
       <c r="I195" s="38" t="s">
-        <v>2042</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="196">
@@ -15621,7 +15661,7 @@
         <v>194</v>
       </c>
       <c r="B196" s="37" t="s">
-        <v>2043</v>
+        <v>2041</v>
       </c>
       <c r="C196" s="37">
         <v>0.0</v>
@@ -15639,10 +15679,10 @@
         <v>777</v>
       </c>
       <c r="H196" s="38" t="s">
-        <v>2044</v>
+        <v>2042</v>
       </c>
       <c r="I196" s="38" t="s">
-        <v>2044</v>
+        <v>2042</v>
       </c>
     </row>
     <row r="197">
@@ -15651,7 +15691,7 @@
         <v>195</v>
       </c>
       <c r="B197" s="37" t="s">
-        <v>2045</v>
+        <v>2043</v>
       </c>
       <c r="C197" s="37">
         <v>0.0</v>
@@ -15669,10 +15709,10 @@
         <v>777</v>
       </c>
       <c r="H197" s="38" t="s">
-        <v>2046</v>
+        <v>2044</v>
       </c>
       <c r="I197" s="38" t="s">
-        <v>2046</v>
+        <v>2044</v>
       </c>
     </row>
     <row r="198">
@@ -15681,7 +15721,7 @@
         <v>196</v>
       </c>
       <c r="B198" s="37" t="s">
-        <v>2047</v>
+        <v>2045</v>
       </c>
       <c r="C198" s="37">
         <v>0.0</v>
@@ -15699,10 +15739,10 @@
         <v>777</v>
       </c>
       <c r="H198" s="38" t="s">
-        <v>2048</v>
+        <v>2046</v>
       </c>
       <c r="I198" s="38" t="s">
-        <v>2048</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="199">
@@ -15711,7 +15751,7 @@
         <v>197</v>
       </c>
       <c r="B199" s="37" t="s">
-        <v>2049</v>
+        <v>2047</v>
       </c>
       <c r="C199" s="37">
         <v>0.0</v>
@@ -15729,10 +15769,10 @@
         <v>777</v>
       </c>
       <c r="H199" s="38" t="s">
-        <v>2050</v>
+        <v>2048</v>
       </c>
       <c r="I199" s="38" t="s">
-        <v>2050</v>
+        <v>2048</v>
       </c>
     </row>
     <row r="200">
@@ -15741,7 +15781,7 @@
         <v>198</v>
       </c>
       <c r="B200" s="37" t="s">
-        <v>2051</v>
+        <v>2049</v>
       </c>
       <c r="C200" s="37">
         <v>1.0</v>
@@ -15759,10 +15799,10 @@
         <v>777</v>
       </c>
       <c r="H200" s="38" t="s">
-        <v>2052</v>
+        <v>2050</v>
       </c>
       <c r="I200" s="38" t="s">
-        <v>2052</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="201">
@@ -15771,7 +15811,7 @@
         <v>199</v>
       </c>
       <c r="B201" s="37" t="s">
-        <v>2053</v>
+        <v>2051</v>
       </c>
       <c r="C201" s="37">
         <v>0.0</v>
@@ -15789,10 +15829,10 @@
         <v>777</v>
       </c>
       <c r="H201" s="38" t="s">
-        <v>2054</v>
+        <v>2052</v>
       </c>
       <c r="I201" s="38" t="s">
-        <v>2054</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="202">
@@ -15801,7 +15841,7 @@
         <v>200</v>
       </c>
       <c r="B202" s="37" t="s">
-        <v>2055</v>
+        <v>2053</v>
       </c>
       <c r="C202" s="37">
         <v>1.0</v>
@@ -15819,10 +15859,10 @@
         <v>777</v>
       </c>
       <c r="H202" s="38" t="s">
-        <v>2056</v>
+        <v>2054</v>
       </c>
       <c r="I202" s="38" t="s">
-        <v>2056</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="203">
@@ -15831,7 +15871,7 @@
         <v>201</v>
       </c>
       <c r="B203" s="37" t="s">
-        <v>2057</v>
+        <v>2055</v>
       </c>
       <c r="C203" s="37">
         <v>0.0</v>
@@ -15849,10 +15889,10 @@
         <v>777</v>
       </c>
       <c r="H203" s="38" t="s">
-        <v>2058</v>
+        <v>2056</v>
       </c>
       <c r="I203" s="38" t="s">
-        <v>2058</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="204">
@@ -15861,7 +15901,7 @@
         <v>202</v>
       </c>
       <c r="B204" s="37" t="s">
-        <v>2059</v>
+        <v>2057</v>
       </c>
       <c r="C204" s="37">
         <v>0.0</v>
@@ -15879,10 +15919,10 @@
         <v>777</v>
       </c>
       <c r="H204" s="38" t="s">
-        <v>2060</v>
+        <v>2058</v>
       </c>
       <c r="I204" s="38" t="s">
-        <v>2060</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="205">
@@ -15891,7 +15931,7 @@
         <v>203</v>
       </c>
       <c r="B205" s="37" t="s">
-        <v>2061</v>
+        <v>2059</v>
       </c>
       <c r="C205" s="37">
         <v>1.0</v>
@@ -15909,10 +15949,10 @@
         <v>777</v>
       </c>
       <c r="H205" s="38" t="s">
-        <v>2062</v>
+        <v>2060</v>
       </c>
       <c r="I205" s="38" t="s">
-        <v>2062</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="206">
@@ -15921,7 +15961,7 @@
         <v>204</v>
       </c>
       <c r="B206" s="37" t="s">
-        <v>2063</v>
+        <v>2061</v>
       </c>
       <c r="C206" s="37">
         <v>0.0</v>
@@ -15939,10 +15979,10 @@
         <v>777</v>
       </c>
       <c r="H206" s="38" t="s">
-        <v>2064</v>
+        <v>2062</v>
       </c>
       <c r="I206" s="38" t="s">
-        <v>2064</v>
+        <v>2062</v>
       </c>
     </row>
     <row r="207">
@@ -15951,7 +15991,7 @@
         <v>205</v>
       </c>
       <c r="B207" s="37" t="s">
-        <v>2065</v>
+        <v>2063</v>
       </c>
       <c r="C207" s="37">
         <v>1.0</v>
@@ -15969,10 +16009,10 @@
         <v>777</v>
       </c>
       <c r="H207" s="38" t="s">
-        <v>2066</v>
+        <v>2064</v>
       </c>
       <c r="I207" s="38" t="s">
-        <v>2066</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="208">
@@ -15981,7 +16021,7 @@
         <v>206</v>
       </c>
       <c r="B208" s="37" t="s">
-        <v>2067</v>
+        <v>2065</v>
       </c>
       <c r="C208" s="37">
         <v>0.0</v>
@@ -15999,10 +16039,10 @@
         <v>777</v>
       </c>
       <c r="H208" s="38" t="s">
-        <v>2068</v>
+        <v>2066</v>
       </c>
       <c r="I208" s="38" t="s">
-        <v>2068</v>
+        <v>2066</v>
       </c>
     </row>
     <row r="209">
@@ -16011,7 +16051,7 @@
         <v>207</v>
       </c>
       <c r="B209" s="37" t="s">
-        <v>2069</v>
+        <v>2067</v>
       </c>
       <c r="C209" s="37">
         <v>1.0</v>
@@ -16029,10 +16069,10 @@
         <v>777</v>
       </c>
       <c r="H209" s="38" t="s">
-        <v>2070</v>
+        <v>2068</v>
       </c>
       <c r="I209" s="38" t="s">
-        <v>2070</v>
+        <v>2068</v>
       </c>
     </row>
     <row r="210">
@@ -16041,7 +16081,7 @@
         <v>208</v>
       </c>
       <c r="B210" s="37" t="s">
-        <v>2071</v>
+        <v>2069</v>
       </c>
       <c r="C210" s="37">
         <v>0.0</v>
@@ -16059,10 +16099,10 @@
         <v>777</v>
       </c>
       <c r="H210" s="38" t="s">
-        <v>2072</v>
+        <v>2070</v>
       </c>
       <c r="I210" s="38" t="s">
-        <v>2072</v>
+        <v>2070</v>
       </c>
     </row>
     <row r="211">
@@ -16071,7 +16111,7 @@
         <v>209</v>
       </c>
       <c r="B211" s="37" t="s">
-        <v>2073</v>
+        <v>2071</v>
       </c>
       <c r="C211" s="37">
         <v>1.0</v>
@@ -16089,10 +16129,10 @@
         <v>777</v>
       </c>
       <c r="H211" s="38" t="s">
-        <v>2074</v>
+        <v>2072</v>
       </c>
       <c r="I211" s="38" t="s">
-        <v>2074</v>
+        <v>2072</v>
       </c>
     </row>
     <row r="212">
@@ -16101,7 +16141,7 @@
         <v>210</v>
       </c>
       <c r="B212" s="37" t="s">
-        <v>2075</v>
+        <v>2073</v>
       </c>
       <c r="C212" s="37">
         <v>0.0</v>
@@ -16119,10 +16159,10 @@
         <v>777</v>
       </c>
       <c r="H212" s="38" t="s">
-        <v>2076</v>
+        <v>2074</v>
       </c>
       <c r="I212" s="38" t="s">
-        <v>2076</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="213">
@@ -16131,7 +16171,7 @@
         <v>211</v>
       </c>
       <c r="B213" s="37" t="s">
-        <v>2077</v>
+        <v>2075</v>
       </c>
       <c r="C213" s="37">
         <v>1.0</v>
@@ -16149,10 +16189,10 @@
         <v>777</v>
       </c>
       <c r="H213" s="38" t="s">
-        <v>2078</v>
+        <v>2076</v>
       </c>
       <c r="I213" s="38" t="s">
-        <v>2078</v>
+        <v>2076</v>
       </c>
     </row>
     <row r="214">
@@ -16161,7 +16201,7 @@
         <v>212</v>
       </c>
       <c r="B214" s="37" t="s">
-        <v>2079</v>
+        <v>2077</v>
       </c>
       <c r="C214" s="37">
         <v>0.0</v>
@@ -16179,10 +16219,10 @@
         <v>777</v>
       </c>
       <c r="H214" s="38" t="s">
-        <v>2080</v>
+        <v>2078</v>
       </c>
       <c r="I214" s="38" t="s">
-        <v>2080</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="215">
@@ -16191,7 +16231,7 @@
         <v>213</v>
       </c>
       <c r="B215" s="37" t="s">
-        <v>2081</v>
+        <v>2079</v>
       </c>
       <c r="C215" s="37">
         <v>1.0</v>
@@ -16209,10 +16249,10 @@
         <v>777</v>
       </c>
       <c r="H215" s="38" t="s">
-        <v>2082</v>
+        <v>2080</v>
       </c>
       <c r="I215" s="38" t="s">
-        <v>2082</v>
+        <v>2080</v>
       </c>
     </row>
     <row r="216">
@@ -16221,7 +16261,7 @@
         <v>214</v>
       </c>
       <c r="B216" s="37" t="s">
-        <v>2083</v>
+        <v>2081</v>
       </c>
       <c r="C216" s="37">
         <v>0.0</v>
@@ -16239,10 +16279,10 @@
         <v>777</v>
       </c>
       <c r="H216" s="38" t="s">
-        <v>2084</v>
+        <v>2082</v>
       </c>
       <c r="I216" s="38" t="s">
-        <v>2084</v>
+        <v>2082</v>
       </c>
     </row>
     <row r="217">
@@ -16251,7 +16291,7 @@
         <v>215</v>
       </c>
       <c r="B217" s="37" t="s">
-        <v>2085</v>
+        <v>2083</v>
       </c>
       <c r="C217" s="37">
         <v>1.0</v>
@@ -16269,10 +16309,10 @@
         <v>777</v>
       </c>
       <c r="H217" s="38" t="s">
-        <v>2086</v>
+        <v>2084</v>
       </c>
       <c r="I217" s="38" t="s">
-        <v>2086</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="218">
@@ -16299,10 +16339,10 @@
         <v>777</v>
       </c>
       <c r="H218" s="38" t="s">
-        <v>2087</v>
+        <v>2085</v>
       </c>
       <c r="I218" s="38" t="s">
-        <v>2087</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="219">
@@ -16311,7 +16351,7 @@
         <v>217</v>
       </c>
       <c r="B219" s="37" t="s">
-        <v>2088</v>
+        <v>2086</v>
       </c>
       <c r="C219" s="37">
         <v>0.0</v>
@@ -16323,16 +16363,16 @@
         <v>1589</v>
       </c>
       <c r="F219" s="39" t="s">
-        <v>2089</v>
+        <v>2087</v>
       </c>
       <c r="G219" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H219" s="38" t="s">
-        <v>2090</v>
+        <v>2088</v>
       </c>
       <c r="I219" s="38" t="s">
-        <v>2090</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="220">
@@ -16341,7 +16381,7 @@
         <v>218</v>
       </c>
       <c r="B220" s="37" t="s">
-        <v>2091</v>
+        <v>2089</v>
       </c>
       <c r="C220" s="37">
         <v>1.0</v>
@@ -16353,16 +16393,16 @@
         <v>1611</v>
       </c>
       <c r="F220" s="39" t="s">
-        <v>2092</v>
+        <v>1589</v>
       </c>
       <c r="G220" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H220" s="38" t="s">
-        <v>2093</v>
+        <v>2090</v>
       </c>
       <c r="I220" s="38" t="s">
-        <v>2093</v>
+        <v>2090</v>
       </c>
     </row>
     <row r="221">
@@ -16371,7 +16411,7 @@
         <v>219</v>
       </c>
       <c r="B221" s="37" t="s">
-        <v>2094</v>
+        <v>2091</v>
       </c>
       <c r="C221" s="37">
         <v>0.0</v>
@@ -16383,16 +16423,16 @@
         <v>1589</v>
       </c>
       <c r="F221" s="39" t="s">
-        <v>2089</v>
+        <v>2087</v>
       </c>
       <c r="G221" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H221" s="38" t="s">
-        <v>2095</v>
+        <v>2092</v>
       </c>
       <c r="I221" s="38" t="s">
-        <v>2095</v>
+        <v>2092</v>
       </c>
     </row>
     <row r="222">
@@ -16401,7 +16441,7 @@
         <v>220</v>
       </c>
       <c r="B222" s="37" t="s">
-        <v>2096</v>
+        <v>2093</v>
       </c>
       <c r="C222" s="37">
         <v>1.0</v>
@@ -16413,16 +16453,16 @@
         <v>1611</v>
       </c>
       <c r="F222" s="39" t="s">
-        <v>2092</v>
+        <v>1589</v>
       </c>
       <c r="G222" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H222" s="38" t="s">
-        <v>2097</v>
+        <v>2094</v>
       </c>
       <c r="I222" s="38" t="s">
-        <v>2097</v>
+        <v>2094</v>
       </c>
     </row>
     <row r="223">
@@ -16431,7 +16471,7 @@
         <v>221</v>
       </c>
       <c r="B223" s="37" t="s">
-        <v>2098</v>
+        <v>2095</v>
       </c>
       <c r="C223" s="37">
         <v>0.0</v>
@@ -16443,16 +16483,16 @@
         <v>1589</v>
       </c>
       <c r="F223" s="39" t="s">
-        <v>2089</v>
+        <v>2087</v>
       </c>
       <c r="G223" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H223" s="38" t="s">
-        <v>2099</v>
+        <v>2096</v>
       </c>
       <c r="I223" s="38" t="s">
-        <v>2099</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="224">
@@ -16461,7 +16501,7 @@
         <v>222</v>
       </c>
       <c r="B224" s="37" t="s">
-        <v>2100</v>
+        <v>2097</v>
       </c>
       <c r="C224" s="37">
         <v>1.0</v>
@@ -16473,16 +16513,16 @@
         <v>1611</v>
       </c>
       <c r="F224" s="39" t="s">
-        <v>2092</v>
+        <v>1589</v>
       </c>
       <c r="G224" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H224" s="38" t="s">
-        <v>2101</v>
+        <v>2098</v>
       </c>
       <c r="I224" s="38" t="s">
-        <v>2101</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="225">
@@ -16503,16 +16543,16 @@
         <v>1589</v>
       </c>
       <c r="F225" s="39" t="s">
-        <v>2089</v>
+        <v>2087</v>
       </c>
       <c r="G225" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H225" s="38" t="s">
-        <v>2102</v>
+        <v>2099</v>
       </c>
       <c r="I225" s="38" t="s">
-        <v>2102</v>
+        <v>2099</v>
       </c>
     </row>
     <row r="226">
@@ -16521,7 +16561,7 @@
         <v>224</v>
       </c>
       <c r="B226" s="37" t="s">
-        <v>2103</v>
+        <v>2100</v>
       </c>
       <c r="C226" s="37">
         <v>1.0</v>
@@ -16533,16 +16573,16 @@
         <v>1611</v>
       </c>
       <c r="F226" s="39" t="s">
-        <v>2092</v>
+        <v>1589</v>
       </c>
       <c r="G226" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H226" s="38" t="s">
-        <v>2104</v>
+        <v>2101</v>
       </c>
       <c r="I226" s="38" t="s">
-        <v>2104</v>
+        <v>2101</v>
       </c>
     </row>
     <row r="227">
@@ -16551,7 +16591,7 @@
         <v>225</v>
       </c>
       <c r="B227" s="37" t="s">
-        <v>2105</v>
+        <v>2102</v>
       </c>
       <c r="C227" s="37">
         <v>0.0</v>
@@ -16563,16 +16603,16 @@
         <v>1589</v>
       </c>
       <c r="F227" s="39" t="s">
-        <v>2089</v>
+        <v>2087</v>
       </c>
       <c r="G227" s="39" t="s">
         <v>777</v>
       </c>
       <c r="H227" s="38" t="s">
-        <v>2106</v>
+        <v>2103</v>
       </c>
       <c r="I227" s="38" t="s">
-        <v>2106</v>
+        <v>2103</v>
       </c>
     </row>
     <row r="228">
@@ -16581,7 +16621,7 @@
         <v>226</v>
       </c>
       <c r="B228" s="37" t="s">
-        <v>2107</v>
+        <v>2104</v>
       </c>
       <c r="C228" s="37">
         <v>0.0</v>
@@ -16599,10 +16639,10 @@
         <v>777</v>
       </c>
       <c r="H228" s="38" t="s">
-        <v>2108</v>
+        <v>2105</v>
       </c>
       <c r="I228" s="38" t="s">
-        <v>2108</v>
+        <v>2105</v>
       </c>
     </row>
   </sheetData>
@@ -16644,34 +16684,34 @@
         <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>2106</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>2107</v>
+      </c>
+      <c r="D1" s="29" t="s">
+        <v>2108</v>
+      </c>
+      <c r="E1" s="29" t="s">
         <v>2109</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="F1" s="29" t="s">
         <v>2110</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="G1" s="29" t="s">
         <v>2111</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="H1" s="29" t="s">
         <v>2112</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="I1" s="29" t="s">
         <v>2113</v>
       </c>
-      <c r="G1" s="29" t="s">
+      <c r="J1" s="64" t="s">
         <v>2114</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="K1" s="64" t="s">
         <v>2115</v>
-      </c>
-      <c r="I1" s="29" t="s">
-        <v>2116</v>
-      </c>
-      <c r="J1" s="64" t="s">
-        <v>2117</v>
-      </c>
-      <c r="K1" s="64" t="s">
-        <v>2118</v>
       </c>
     </row>
     <row r="2" ht="186.0" customHeight="1">
@@ -16680,7 +16720,7 @@
         <v>-1</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>2119</v>
+        <v>2116</v>
       </c>
       <c r="C2" s="66" t="s">
         <v>338</v>
@@ -16716,7 +16756,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>2120</v>
+        <v>2117</v>
       </c>
       <c r="C3" s="66" t="s">
         <v>982</v>
@@ -16725,10 +16765,10 @@
         <v>1083</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>2122</v>
+        <v>2119</v>
       </c>
       <c r="G3" s="36" t="s">
         <v>336</v>
@@ -16752,19 +16792,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>2123</v>
+        <v>2120</v>
       </c>
       <c r="C4" s="66" t="s">
-        <v>2124</v>
+        <v>2121</v>
       </c>
       <c r="D4" s="67" t="s">
         <v>1083</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>2124</v>
+        <v>2121</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>2125</v>
+        <v>2122</v>
       </c>
       <c r="G4" s="36" t="s">
         <v>336</v>
@@ -16788,19 +16828,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>2126</v>
+        <v>2123</v>
       </c>
       <c r="C5" s="66" t="s">
-        <v>2127</v>
+        <v>2124</v>
       </c>
       <c r="D5" s="67" t="s">
         <v>1083</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>2127</v>
+        <v>2124</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>2128</v>
+        <v>2125</v>
       </c>
       <c r="G5" s="36" t="s">
         <v>336</v>
@@ -16824,19 +16864,19 @@
         <v>3</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
       <c r="C6" s="66" t="s">
-        <v>2130</v>
+        <v>2127</v>
       </c>
       <c r="D6" s="67" t="s">
         <v>1083</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>2130</v>
+        <v>2127</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>2131</v>
+        <v>2128</v>
       </c>
       <c r="G6" s="36" t="s">
         <v>336</v>
@@ -16860,25 +16900,25 @@
         <v>4</v>
       </c>
       <c r="B7" s="30" t="s">
+        <v>2129</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>2130</v>
+      </c>
+      <c r="D7" s="67" t="s">
+        <v>2131</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>2130</v>
+      </c>
+      <c r="F7" s="36" t="s">
         <v>2132</v>
-      </c>
-      <c r="C7" s="33" t="s">
-        <v>2133</v>
-      </c>
-      <c r="D7" s="67" t="s">
-        <v>2134</v>
-      </c>
-      <c r="E7" s="36" t="s">
-        <v>2133</v>
-      </c>
-      <c r="F7" s="36" t="s">
-        <v>2135</v>
       </c>
       <c r="G7" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H7" s="36" t="s">
-        <v>2134</v>
+        <v>2131</v>
       </c>
       <c r="I7" s="36" t="s">
         <v>682</v>
@@ -16896,25 +16936,25 @@
         <v>5</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>2136</v>
+        <v>2133</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>2137</v>
+        <v>2134</v>
       </c>
       <c r="D8" s="67" t="s">
+        <v>2131</v>
+      </c>
+      <c r="E8" s="36" t="s">
         <v>2134</v>
       </c>
-      <c r="E8" s="36" t="s">
-        <v>2137</v>
-      </c>
       <c r="F8" s="36" t="s">
-        <v>2138</v>
+        <v>2135</v>
       </c>
       <c r="G8" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H8" s="36" t="s">
-        <v>2134</v>
+        <v>2131</v>
       </c>
       <c r="I8" s="36" t="s">
         <v>682</v>
@@ -16932,7 +16972,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>2139</v>
+        <v>2136</v>
       </c>
       <c r="C9" s="33" t="s">
         <v>1019</v>
@@ -16944,7 +16984,7 @@
         <v>1019</v>
       </c>
       <c r="F9" s="36" t="s">
-        <v>2140</v>
+        <v>2137</v>
       </c>
       <c r="G9" s="36" t="s">
         <v>336</v>
@@ -16968,25 +17008,25 @@
         <v>7</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>2141</v>
+        <v>2138</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
       <c r="D10" s="67" t="s">
         <v>1079</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>2142</v>
+        <v>2139</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>2143</v>
+        <v>2140</v>
       </c>
       <c r="G10" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>2144</v>
+        <v>2141</v>
       </c>
       <c r="I10" s="36" t="s">
         <v>745</v>
@@ -17004,25 +17044,25 @@
         <v>8</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>2145</v>
+        <v>2142</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
       <c r="D11" s="67" t="s">
-        <v>2134</v>
+        <v>2131</v>
       </c>
       <c r="E11" s="36" t="s">
-        <v>2146</v>
+        <v>2143</v>
       </c>
       <c r="F11" s="36" t="s">
-        <v>2147</v>
+        <v>2144</v>
       </c>
       <c r="G11" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H11" s="36" t="s">
-        <v>2148</v>
+        <v>2145</v>
       </c>
       <c r="I11" s="36" t="s">
         <v>682</v>
@@ -17040,19 +17080,19 @@
         <v>9</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>2149</v>
+        <v>2146</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>2150</v>
+        <v>2147</v>
       </c>
       <c r="D12" s="67" t="s">
         <v>1078</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>2150</v>
+        <v>2147</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>2151</v>
+        <v>2148</v>
       </c>
       <c r="G12" s="36" t="s">
         <v>336</v>
@@ -17076,25 +17116,25 @@
         <v>10</v>
       </c>
       <c r="B13" s="30" t="s">
+        <v>2149</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>2150</v>
+      </c>
+      <c r="D13" s="67" t="s">
+        <v>2151</v>
+      </c>
+      <c r="E13" s="36" t="s">
+        <v>2150</v>
+      </c>
+      <c r="F13" s="36" t="s">
         <v>2152</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>2153</v>
-      </c>
-      <c r="D13" s="67" t="s">
-        <v>2154</v>
-      </c>
-      <c r="E13" s="36" t="s">
-        <v>2153</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>2155</v>
       </c>
       <c r="G13" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>2156</v>
+        <v>2153</v>
       </c>
       <c r="I13" s="36" t="s">
         <v>682</v>
@@ -17121,16 +17161,16 @@
         <v>22</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>2157</v>
+        <v>2154</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>2158</v>
+        <v>2155</v>
       </c>
       <c r="G14" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>2159</v>
+        <v>2156</v>
       </c>
       <c r="I14" s="36" t="s">
         <v>682</v>
@@ -17157,16 +17197,16 @@
         <v>22</v>
       </c>
       <c r="E15" s="36" t="s">
-        <v>2160</v>
+        <v>2157</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>2161</v>
+        <v>2158</v>
       </c>
       <c r="G15" s="36" t="s">
         <v>336</v>
       </c>
       <c r="H15" s="36" t="s">
-        <v>2162</v>
+        <v>2159</v>
       </c>
       <c r="I15" s="36" t="s">
         <v>682</v>
@@ -17184,7 +17224,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>2163</v>
+        <v>2160</v>
       </c>
       <c r="C16" s="66" t="s">
         <v>338</v>
@@ -17236,7 +17276,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="44.0"/>
-    <col customWidth="1" min="3" max="3" width="38.86"/>
+    <col customWidth="1" min="3" max="3" width="63.14"/>
     <col customWidth="1" min="4" max="4" width="23.29"/>
     <col customWidth="1" min="6" max="6" width="38.86"/>
     <col customWidth="1" min="8" max="8" width="34.57"/>
@@ -17247,7 +17287,7 @@
         <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2164</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="2">
@@ -17274,7 +17314,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>2165</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="5">
@@ -17283,7 +17323,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>2166</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="6">
@@ -17295,7 +17335,7 @@
         <v>51</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>2167</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="8">
@@ -17303,7 +17343,7 @@
         <v>0.0</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>2168</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="9">
@@ -17311,7 +17351,7 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>2169</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="10">
@@ -17319,7 +17359,7 @@
         <v>2.0</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>2170</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="11">
@@ -17327,7 +17367,7 @@
         <v>3.0</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>2171</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="12">
@@ -17335,7 +17375,7 @@
         <v>4.0</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>2172</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="13">
@@ -17343,7 +17383,7 @@
         <v>5.0</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>2173</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="15">
@@ -17351,7 +17391,7 @@
         <v>51</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>2174</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="16">
@@ -17369,7 +17409,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>2175</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="18">
@@ -17414,7 +17454,7 @@
         <v>6</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>2176</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="23">
@@ -17431,7 +17471,7 @@
         <v>51</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>2177</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="26">
@@ -17476,7 +17516,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>2178</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="31">
@@ -17512,7 +17552,7 @@
         <v>8</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>2179</v>
+        <v>2176</v>
       </c>
     </row>
     <row r="35">
@@ -17530,7 +17570,7 @@
         <v>10</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>2180</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="37">
@@ -17601,7 +17641,10 @@
         <v>51</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>2181</v>
+        <v>2178</v>
+      </c>
+      <c r="C45" s="47" t="s">
+        <v>2179</v>
       </c>
     </row>
     <row r="46">
@@ -17612,6 +17655,9 @@
       <c r="B46" s="37" t="s">
         <v>777</v>
       </c>
+      <c r="C46" s="37" t="s">
+        <v>2180</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="37">
@@ -17619,7 +17665,10 @@
         <v>1</v>
       </c>
       <c r="B47" s="37" t="s">
-        <v>1974</v>
+        <v>1972</v>
+      </c>
+      <c r="C47" s="37" t="s">
+        <v>2181</v>
       </c>
     </row>
     <row r="48">
@@ -17628,7 +17677,7 @@
         <v>2</v>
       </c>
       <c r="B48" s="37" t="s">
-        <v>1927</v>
+        <v>956</v>
       </c>
     </row>
     <row r="49">
@@ -17637,7 +17686,7 @@
         <v>3</v>
       </c>
       <c r="B49" s="37" t="s">
-        <v>1920</v>
+        <v>960</v>
       </c>
     </row>
     <row r="50">
@@ -17646,7 +17695,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="37" t="s">
-        <v>1936</v>
+        <v>1934</v>
       </c>
     </row>
     <row r="51">
@@ -17693,6 +17742,9 @@
       <c r="B55" s="37" t="s">
         <v>2186</v>
       </c>
+      <c r="C55" s="37" t="s">
+        <v>2187</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="37">
@@ -17709,7 +17761,7 @@
         <v>11</v>
       </c>
       <c r="B57" s="37" t="s">
-        <v>2187</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="58">
@@ -17718,7 +17770,7 @@
         <v>12</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>2188</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="59">
@@ -17727,7 +17779,7 @@
         <v>13</v>
       </c>
       <c r="B59" s="37" t="s">
-        <v>1611</v>
+        <v>2190</v>
       </c>
     </row>
     <row r="60">
@@ -17736,7 +17788,7 @@
         <v>14</v>
       </c>
       <c r="B60" s="37" t="s">
-        <v>1589</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="61">
@@ -17745,7 +17797,7 @@
         <v>15</v>
       </c>
       <c r="B61" s="37" t="s">
-        <v>960</v>
+        <v>2192</v>
       </c>
     </row>
     <row r="62">
@@ -17754,7 +17806,7 @@
         <v>16</v>
       </c>
       <c r="B62" s="37" t="s">
-        <v>956</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="63">
@@ -17763,7 +17815,7 @@
         <v>17</v>
       </c>
       <c r="B63" s="37" t="s">
-        <v>2089</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="64">
@@ -17772,7 +17824,7 @@
         <v>18</v>
       </c>
       <c r="B64" s="37" t="s">
-        <v>2092</v>
+        <v>2087</v>
       </c>
     </row>
     <row r="65">
@@ -17781,7 +17833,7 @@
         <v>19</v>
       </c>
       <c r="B65" s="37" t="s">
-        <v>2189</v>
+        <v>2194</v>
       </c>
     </row>
     <row r="66">
@@ -17790,7 +17842,7 @@
         <v>20</v>
       </c>
       <c r="B66" s="37" t="s">
-        <v>2190</v>
+        <v>2195</v>
       </c>
     </row>
     <row r="67">
@@ -17799,7 +17851,10 @@
         <v>21</v>
       </c>
       <c r="B67" s="37" t="s">
-        <v>2191</v>
+        <v>1589</v>
+      </c>
+      <c r="C67" s="37" t="s">
+        <v>2196</v>
       </c>
     </row>
     <row r="68">
@@ -17808,7 +17863,7 @@
         <v>22</v>
       </c>
       <c r="B68" s="37" t="s">
-        <v>2192</v>
+        <v>2197</v>
       </c>
     </row>
     <row r="69">
@@ -17817,7 +17872,7 @@
         <v>23</v>
       </c>
       <c r="B69" s="37" t="s">
-        <v>2193</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="70">
@@ -17826,94 +17881,154 @@
         <v>24</v>
       </c>
       <c r="B70" s="37" t="s">
-        <v>2194</v>
+        <v>2199</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="37">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>25</v>
+      </c>
+      <c r="B71" s="37" t="s">
+        <v>2200</v>
+      </c>
+      <c r="C71" s="37" t="s">
+        <v>2201</v>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>2195</v>
+      <c r="A72" s="37">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>26</v>
+      </c>
+      <c r="B72" s="37" t="s">
+        <v>2202</v>
+      </c>
+      <c r="C72" s="37" t="s">
+        <v>2203</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="37">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>27</v>
+      </c>
+      <c r="B73" s="37" t="s">
+        <v>2204</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="37">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>28</v>
+      </c>
+      <c r="B74" s="37" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="37">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>29</v>
+      </c>
+      <c r="B75" s="37" t="s">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="37">
+        <f>ROW()-ROW(Table_Animation_Trigger[N])</f>
+        <v>30</v>
+      </c>
+      <c r="B76" s="37" t="s">
+        <v>2207</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="37">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>0</v>
       </c>
-      <c r="B73" s="37" t="s">
+      <c r="B79" s="37" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="37">
+    <row r="80">
+      <c r="A80" s="37">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>1</v>
       </c>
-      <c r="B74" s="37" t="s">
+      <c r="B80" s="37" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="37">
+    <row r="81">
+      <c r="A81" s="37">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>2</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B81" s="1" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="37">
+    <row r="82">
+      <c r="A82" s="37">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>3</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B82" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="37">
+    <row r="83">
+      <c r="A83" s="37">
         <f>ROW()-ROW(Table_Item_Family_Type[N])</f>
         <v>4</v>
       </c>
-      <c r="B77" s="68" t="s">
+      <c r="B83" s="68" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="1" t="s">
+    <row r="85">
+      <c r="A85" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B79" s="1" t="s">
-        <v>2196</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="37">
+      <c r="B85" s="1" t="s">
+        <v>2209</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="37">
         <f>ROW()-ROW(Table_Moment_Day[N])</f>
         <v>0</v>
       </c>
-      <c r="B80" s="37" t="s">
+      <c r="B86" s="37" t="s">
         <v>572</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="37">
+    <row r="87">
+      <c r="A87" s="37">
         <f>ROW()-ROW(Table_Moment_Day[N])</f>
         <v>1</v>
       </c>
-      <c r="B81" s="37" t="s">
+      <c r="B87" s="37" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="37">
+    <row r="88">
+      <c r="A88" s="37">
         <f>ROW()-ROW(Table_Moment_Day[N])</f>
         <v>2</v>
       </c>
-      <c r="B82" s="37" t="s">
+      <c r="B88" s="37" t="s">
         <v>510</v>
       </c>
     </row>
@@ -17952,7 +18067,7 @@
         <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2197</v>
+        <v>2210</v>
       </c>
     </row>
     <row r="2">
@@ -17970,7 +18085,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>2198</v>
+        <v>2211</v>
       </c>
     </row>
     <row r="4">
@@ -17979,7 +18094,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>2199</v>
+        <v>2212</v>
       </c>
     </row>
     <row r="5">
@@ -18060,7 +18175,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>2200</v>
+        <v>2213</v>
       </c>
     </row>
     <row r="14">
@@ -18105,7 +18220,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>2201</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="19">
@@ -18294,7 +18409,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>2202</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="40">
@@ -18312,7 +18427,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="37" t="s">
-        <v>2203</v>
+        <v>2216</v>
       </c>
     </row>
     <row r="43">
@@ -18320,16 +18435,16 @@
         <v>51</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>2204</v>
+        <v>2217</v>
       </c>
       <c r="C43" s="69" t="s">
         <v>327</v>
       </c>
       <c r="D43" s="69" t="s">
-        <v>2205</v>
+        <v>2218</v>
       </c>
       <c r="E43" s="69" t="s">
-        <v>2206</v>
+        <v>2219</v>
       </c>
     </row>
     <row r="44">
@@ -18338,7 +18453,7 @@
         <v>0</v>
       </c>
       <c r="B44" s="37" t="s">
-        <v>2207</v>
+        <v>2220</v>
       </c>
       <c r="C44" s="39" t="s">
         <v>336</v>
@@ -18357,7 +18472,7 @@
         <v>1</v>
       </c>
       <c r="B45" s="37" t="s">
-        <v>2208</v>
+        <v>2221</v>
       </c>
       <c r="C45" s="39" t="s">
         <v>1510</v>
@@ -18376,7 +18491,7 @@
         <v>2</v>
       </c>
       <c r="B46" s="37" t="s">
-        <v>2209</v>
+        <v>2222</v>
       </c>
       <c r="C46" s="39" t="s">
         <v>1541</v>
@@ -18414,7 +18529,7 @@
         <v>4</v>
       </c>
       <c r="B48" s="37" t="s">
-        <v>2210</v>
+        <v>2223</v>
       </c>
       <c r="C48" s="39" t="s">
         <v>500</v>
@@ -18432,19 +18547,19 @@
         <v>51</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>2211</v>
+        <v>2224</v>
       </c>
       <c r="C50" s="68" t="s">
-        <v>2212</v>
+        <v>2225</v>
       </c>
       <c r="D50" s="68" t="s">
         <v>1473</v>
       </c>
       <c r="E50" s="69" t="s">
-        <v>2213</v>
+        <v>2226</v>
       </c>
       <c r="F50" s="68" t="s">
-        <v>2214</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="51">
@@ -18456,13 +18571,13 @@
         <v>773</v>
       </c>
       <c r="C51" s="45" t="s">
-        <v>2207</v>
+        <v>2220</v>
       </c>
       <c r="D51" s="45" t="s">
         <v>776</v>
       </c>
       <c r="E51" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F51" s="44" t="b">
         <v>0</v>
@@ -18477,13 +18592,13 @@
         <v>787</v>
       </c>
       <c r="C52" s="45" t="s">
-        <v>2208</v>
+        <v>2221</v>
       </c>
       <c r="D52" s="45" t="s">
         <v>1630</v>
       </c>
       <c r="E52" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F52" s="44" t="b">
         <v>0</v>
@@ -18498,13 +18613,13 @@
         <v>804</v>
       </c>
       <c r="C53" s="45" t="s">
-        <v>2208</v>
+        <v>2221</v>
       </c>
       <c r="D53" s="45" t="s">
         <v>824</v>
       </c>
       <c r="E53" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F53" s="44" t="b">
         <v>0</v>
@@ -18519,13 +18634,13 @@
         <v>809</v>
       </c>
       <c r="C54" s="45" t="s">
-        <v>2209</v>
+        <v>2222</v>
       </c>
       <c r="D54" s="45" t="s">
         <v>1732</v>
       </c>
       <c r="E54" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F54" s="44" t="b">
         <v>0</v>
@@ -18546,7 +18661,7 @@
         <v>1805</v>
       </c>
       <c r="E55" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F55" s="44" t="b">
         <v>0</v>
@@ -18558,7 +18673,7 @@
         <v>5</v>
       </c>
       <c r="B56" s="37" t="s">
-        <v>2216</v>
+        <v>2229</v>
       </c>
       <c r="C56" s="45" t="s">
         <v>46</v>
@@ -18567,7 +18682,7 @@
         <v>1808</v>
       </c>
       <c r="E56" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F56" s="44" t="b">
         <v>0</v>
@@ -18579,7 +18694,7 @@
         <v>6</v>
       </c>
       <c r="B57" s="37" t="s">
-        <v>2217</v>
+        <v>2230</v>
       </c>
       <c r="C57" s="45" t="s">
         <v>46</v>
@@ -18588,7 +18703,7 @@
         <v>1811</v>
       </c>
       <c r="E57" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F57" s="44" t="b">
         <v>1</v>
@@ -18600,16 +18715,16 @@
         <v>7</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>2218</v>
+        <v>2231</v>
       </c>
       <c r="C58" s="45" t="s">
-        <v>2210</v>
+        <v>2223</v>
       </c>
       <c r="D58" s="45" t="s">
         <v>776</v>
       </c>
       <c r="E58" s="49" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="F58" s="44" t="b">
         <v>0</v>
@@ -18620,10 +18735,10 @@
         <v>51</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>2219</v>
+        <v>2232</v>
       </c>
       <c r="C60" s="29" t="s">
-        <v>2220</v>
+        <v>2233</v>
       </c>
     </row>
     <row r="61">
@@ -18632,7 +18747,7 @@
         <v>0</v>
       </c>
       <c r="B61" s="37" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="C61" s="52" t="s">
         <v>509</v>
@@ -18643,7 +18758,7 @@
         <v>51</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>2221</v>
+        <v>2234</v>
       </c>
     </row>
     <row r="64">
@@ -19695,16 +19810,16 @@
         <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2222</v>
+        <v>2235</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2223</v>
+        <v>2236</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2224</v>
+        <v>2237</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2225</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="2">
@@ -19716,7 +19831,7 @@
         <v>339</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>2226</v>
+        <v>2239</v>
       </c>
       <c r="D2" s="71" t="s">
         <v>336</v>
@@ -19734,7 +19849,7 @@
         <v>454</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>2227</v>
+        <v>2240</v>
       </c>
       <c r="D3" s="71" t="s">
         <v>336</v>
@@ -19749,10 +19864,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>2228</v>
+        <v>2241</v>
       </c>
       <c r="C4" s="30" t="s">
-        <v>2226</v>
+        <v>2239</v>
       </c>
       <c r="D4" s="71" t="s">
         <v>336</v>
@@ -19790,7 +19905,7 @@
         <v>51</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2167</v>
+        <v>2164</v>
       </c>
     </row>
     <row r="2">
@@ -19817,7 +19932,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>2229</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="6">
@@ -19825,7 +19940,7 @@
         <v>51</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>2230</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="7">
@@ -19870,21 +19985,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>2231</v>
+        <v>2244</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2232</v>
+        <v>2245</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2233</v>
+        <v>2246</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2234</v>
+        <v>2247</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="38" t="s">
-        <v>2235</v>
+        <v>2248</v>
       </c>
       <c r="B2" s="72">
         <v>5.0</v>
@@ -19898,7 +20013,7 @@
     </row>
     <row r="3">
       <c r="A3" s="38" t="s">
-        <v>2236</v>
+        <v>2249</v>
       </c>
       <c r="B3" s="72">
         <v>4.0</v>
@@ -19912,7 +20027,7 @@
     </row>
     <row r="4">
       <c r="A4" s="38" t="s">
-        <v>2237</v>
+        <v>2250</v>
       </c>
       <c r="B4" s="72">
         <v>2.0</v>
@@ -19926,7 +20041,7 @@
     </row>
     <row r="5">
       <c r="A5" s="38" t="s">
-        <v>2238</v>
+        <v>2251</v>
       </c>
       <c r="B5" s="72">
         <v>5.0</v>
@@ -19940,7 +20055,7 @@
     </row>
     <row r="6">
       <c r="A6" s="38" t="s">
-        <v>2239</v>
+        <v>2252</v>
       </c>
       <c r="B6" s="72">
         <v>4.0</v>
@@ -19954,7 +20069,7 @@
     </row>
     <row r="7">
       <c r="A7" s="38" t="s">
-        <v>2240</v>
+        <v>2253</v>
       </c>
       <c r="B7" s="72">
         <v>4.0</v>
@@ -19968,7 +20083,7 @@
     </row>
     <row r="8">
       <c r="A8" s="38" t="s">
-        <v>2241</v>
+        <v>2254</v>
       </c>
       <c r="B8" s="72">
         <v>2.0</v>
@@ -26886,9 +27001,8 @@
     <col customWidth="1" min="9" max="9" width="58.57"/>
     <col customWidth="1" min="10" max="10" width="71.14"/>
     <col customWidth="1" min="11" max="11" width="54.43"/>
-    <col customWidth="1" min="12" max="12" width="71.14"/>
-    <col customWidth="1" min="13" max="13" width="24.71"/>
-    <col customWidth="1" min="14" max="14" width="34.14"/>
+    <col customWidth="1" min="12" max="13" width="71.14"/>
+    <col customWidth="1" min="14" max="14" width="45.86"/>
     <col customWidth="1" min="15" max="15" width="30.43"/>
     <col customWidth="1" min="16" max="16" width="25.57"/>
   </cols>
@@ -37029,7 +37143,7 @@
       <c r="M248" s="53" t="s">
         <v>776</v>
       </c>
-      <c r="N248" s="53" t="s">
+      <c r="N248" s="45" t="s">
         <v>777</v>
       </c>
       <c r="O248" s="53" t="s">
@@ -37437,7 +37551,7 @@
       <c r="M256" s="53" t="s">
         <v>776</v>
       </c>
-      <c r="N256" s="53" t="s">
+      <c r="N256" s="45" t="s">
         <v>777</v>
       </c>
       <c r="O256" s="53" t="s">
@@ -37692,7 +37806,7 @@
       <c r="M261" s="53" t="s">
         <v>776</v>
       </c>
-      <c r="N261" s="53" t="s">
+      <c r="N261" s="45" t="s">
         <v>777</v>
       </c>
       <c r="O261" s="53" t="s">

</xml_diff>

<commit_message>
New animations for character
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -17381,10 +17381,10 @@
         <v>1683</v>
       </c>
       <c r="F240" s="45" t="s">
-        <v>964</v>
+        <v>806</v>
       </c>
       <c r="G240" s="45" t="s">
-        <v>964</v>
+        <v>806</v>
       </c>
       <c r="H240" s="42" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
Fix in animations comming out from steady state
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -6536,6 +6536,9 @@
     <t>PHRASE_DIALOG_CLOWN_EXTRAPERLO_OPTION_1_1</t>
   </si>
   <si>
+    <t>ANIMATION_TRIGGER_CYCLE_ONE</t>
+  </si>
+  <si>
     <t>No hombre no... El payaso se lleva dentro. No hay nada más lamentable de ver a un profesional despojado de su hábito. Haciendo la compra y cosas mundanas. La gente te pierde el respeto.</t>
   </si>
   <si>
@@ -7005,9 +7008,6 @@
   </si>
   <si>
     <t>ANIMATION_TRIGGER_EIGHT</t>
-  </si>
-  <si>
-    <t>ANIMATION_TRIGGER_CYCLE_ONE</t>
   </si>
   <si>
     <t>Cycles talk and walk have substeps inside</t>
@@ -16178,7 +16178,7 @@
         <v>1294</v>
       </c>
       <c r="E200" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F200" s="39" t="s">
         <v>1691</v>
@@ -16187,10 +16187,10 @@
         <v>806</v>
       </c>
       <c r="H200" s="38" t="s">
-        <v>2144</v>
+        <v>2145</v>
       </c>
       <c r="I200" s="38" t="s">
-        <v>2144</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="201">
@@ -16199,7 +16199,7 @@
         <v>199</v>
       </c>
       <c r="B201" s="37" t="s">
-        <v>2145</v>
+        <v>2146</v>
       </c>
       <c r="C201" s="37">
         <v>0.0</v>
@@ -16217,10 +16217,10 @@
         <v>806</v>
       </c>
       <c r="H201" s="38" t="s">
-        <v>2146</v>
+        <v>2147</v>
       </c>
       <c r="I201" s="38" t="s">
-        <v>2146</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="202">
@@ -16229,7 +16229,7 @@
         <v>200</v>
       </c>
       <c r="B202" s="37" t="s">
-        <v>2147</v>
+        <v>2148</v>
       </c>
       <c r="C202" s="37">
         <v>1.0</v>
@@ -16238,7 +16238,7 @@
         <v>1298</v>
       </c>
       <c r="E202" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F202" s="39" t="s">
         <v>1691</v>
@@ -16247,10 +16247,10 @@
         <v>806</v>
       </c>
       <c r="H202" s="38" t="s">
-        <v>2148</v>
+        <v>2149</v>
       </c>
       <c r="I202" s="38" t="s">
-        <v>2148</v>
+        <v>2149</v>
       </c>
     </row>
     <row r="203">
@@ -16259,7 +16259,7 @@
         <v>201</v>
       </c>
       <c r="B203" s="37" t="s">
-        <v>2149</v>
+        <v>2150</v>
       </c>
       <c r="C203" s="37">
         <v>0.0</v>
@@ -16277,10 +16277,10 @@
         <v>806</v>
       </c>
       <c r="H203" s="38" t="s">
-        <v>2150</v>
+        <v>2151</v>
       </c>
       <c r="I203" s="38" t="s">
-        <v>2150</v>
+        <v>2151</v>
       </c>
     </row>
     <row r="204">
@@ -16289,7 +16289,7 @@
         <v>202</v>
       </c>
       <c r="B204" s="37" t="s">
-        <v>2151</v>
+        <v>2152</v>
       </c>
       <c r="C204" s="37">
         <v>0.0</v>
@@ -16307,10 +16307,10 @@
         <v>806</v>
       </c>
       <c r="H204" s="38" t="s">
-        <v>2152</v>
+        <v>2153</v>
       </c>
       <c r="I204" s="38" t="s">
-        <v>2152</v>
+        <v>2153</v>
       </c>
     </row>
     <row r="205">
@@ -16319,7 +16319,7 @@
         <v>203</v>
       </c>
       <c r="B205" s="37" t="s">
-        <v>2153</v>
+        <v>2154</v>
       </c>
       <c r="C205" s="37">
         <v>1.0</v>
@@ -16328,7 +16328,7 @@
         <v>1304</v>
       </c>
       <c r="E205" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F205" s="39" t="s">
         <v>1691</v>
@@ -16337,10 +16337,10 @@
         <v>806</v>
       </c>
       <c r="H205" s="38" t="s">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="I205" s="38" t="s">
-        <v>2154</v>
+        <v>2155</v>
       </c>
     </row>
     <row r="206">
@@ -16349,7 +16349,7 @@
         <v>204</v>
       </c>
       <c r="B206" s="37" t="s">
-        <v>2155</v>
+        <v>2156</v>
       </c>
       <c r="C206" s="37">
         <v>0.0</v>
@@ -16367,10 +16367,10 @@
         <v>806</v>
       </c>
       <c r="H206" s="38" t="s">
-        <v>2156</v>
+        <v>2157</v>
       </c>
       <c r="I206" s="38" t="s">
-        <v>2156</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="207">
@@ -16379,7 +16379,7 @@
         <v>205</v>
       </c>
       <c r="B207" s="37" t="s">
-        <v>2157</v>
+        <v>2158</v>
       </c>
       <c r="C207" s="37">
         <v>1.0</v>
@@ -16388,7 +16388,7 @@
         <v>1308</v>
       </c>
       <c r="E207" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F207" s="39" t="s">
         <v>1691</v>
@@ -16397,10 +16397,10 @@
         <v>806</v>
       </c>
       <c r="H207" s="38" t="s">
-        <v>2158</v>
+        <v>2159</v>
       </c>
       <c r="I207" s="38" t="s">
-        <v>2158</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="208">
@@ -16409,7 +16409,7 @@
         <v>206</v>
       </c>
       <c r="B208" s="37" t="s">
-        <v>2159</v>
+        <v>2160</v>
       </c>
       <c r="C208" s="37">
         <v>0.0</v>
@@ -16427,10 +16427,10 @@
         <v>806</v>
       </c>
       <c r="H208" s="38" t="s">
-        <v>2160</v>
+        <v>2161</v>
       </c>
       <c r="I208" s="38" t="s">
-        <v>2160</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="209">
@@ -16439,7 +16439,7 @@
         <v>207</v>
       </c>
       <c r="B209" s="37" t="s">
-        <v>2161</v>
+        <v>2162</v>
       </c>
       <c r="C209" s="37">
         <v>1.0</v>
@@ -16448,7 +16448,7 @@
         <v>1312</v>
       </c>
       <c r="E209" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F209" s="39" t="s">
         <v>1691</v>
@@ -16457,10 +16457,10 @@
         <v>806</v>
       </c>
       <c r="H209" s="38" t="s">
-        <v>2162</v>
+        <v>2163</v>
       </c>
       <c r="I209" s="38" t="s">
-        <v>2162</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="210">
@@ -16469,7 +16469,7 @@
         <v>208</v>
       </c>
       <c r="B210" s="37" t="s">
-        <v>2163</v>
+        <v>2164</v>
       </c>
       <c r="C210" s="37">
         <v>0.0</v>
@@ -16487,10 +16487,10 @@
         <v>806</v>
       </c>
       <c r="H210" s="38" t="s">
-        <v>2164</v>
+        <v>2165</v>
       </c>
       <c r="I210" s="38" t="s">
-        <v>2164</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="211">
@@ -16499,7 +16499,7 @@
         <v>209</v>
       </c>
       <c r="B211" s="37" t="s">
-        <v>2165</v>
+        <v>2166</v>
       </c>
       <c r="C211" s="37">
         <v>1.0</v>
@@ -16508,7 +16508,7 @@
         <v>1316</v>
       </c>
       <c r="E211" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F211" s="39" t="s">
         <v>1691</v>
@@ -16517,10 +16517,10 @@
         <v>806</v>
       </c>
       <c r="H211" s="38" t="s">
-        <v>2166</v>
+        <v>2167</v>
       </c>
       <c r="I211" s="38" t="s">
-        <v>2166</v>
+        <v>2167</v>
       </c>
     </row>
     <row r="212">
@@ -16529,7 +16529,7 @@
         <v>210</v>
       </c>
       <c r="B212" s="37" t="s">
-        <v>2167</v>
+        <v>2168</v>
       </c>
       <c r="C212" s="37">
         <v>0.0</v>
@@ -16547,10 +16547,10 @@
         <v>806</v>
       </c>
       <c r="H212" s="38" t="s">
-        <v>2168</v>
+        <v>2169</v>
       </c>
       <c r="I212" s="38" t="s">
-        <v>2168</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="213">
@@ -16559,7 +16559,7 @@
         <v>211</v>
       </c>
       <c r="B213" s="37" t="s">
-        <v>2169</v>
+        <v>2170</v>
       </c>
       <c r="C213" s="37">
         <v>1.0</v>
@@ -16568,7 +16568,7 @@
         <v>1320</v>
       </c>
       <c r="E213" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F213" s="39" t="s">
         <v>1691</v>
@@ -16577,10 +16577,10 @@
         <v>806</v>
       </c>
       <c r="H213" s="38" t="s">
-        <v>2170</v>
+        <v>2171</v>
       </c>
       <c r="I213" s="38" t="s">
-        <v>2170</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="214">
@@ -16589,7 +16589,7 @@
         <v>212</v>
       </c>
       <c r="B214" s="37" t="s">
-        <v>2171</v>
+        <v>2172</v>
       </c>
       <c r="C214" s="37">
         <v>0.0</v>
@@ -16607,10 +16607,10 @@
         <v>806</v>
       </c>
       <c r="H214" s="38" t="s">
-        <v>2172</v>
+        <v>2173</v>
       </c>
       <c r="I214" s="38" t="s">
-        <v>2172</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="215">
@@ -16619,7 +16619,7 @@
         <v>213</v>
       </c>
       <c r="B215" s="37" t="s">
-        <v>2173</v>
+        <v>2174</v>
       </c>
       <c r="C215" s="37">
         <v>1.0</v>
@@ -16628,7 +16628,7 @@
         <v>1324</v>
       </c>
       <c r="E215" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F215" s="39" t="s">
         <v>1691</v>
@@ -16637,10 +16637,10 @@
         <v>806</v>
       </c>
       <c r="H215" s="38" t="s">
-        <v>2174</v>
+        <v>2175</v>
       </c>
       <c r="I215" s="38" t="s">
-        <v>2174</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="216">
@@ -16649,7 +16649,7 @@
         <v>214</v>
       </c>
       <c r="B216" s="37" t="s">
-        <v>2175</v>
+        <v>2176</v>
       </c>
       <c r="C216" s="37">
         <v>0.0</v>
@@ -16667,10 +16667,10 @@
         <v>806</v>
       </c>
       <c r="H216" s="38" t="s">
-        <v>2176</v>
+        <v>2177</v>
       </c>
       <c r="I216" s="38" t="s">
-        <v>2176</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="217">
@@ -16679,7 +16679,7 @@
         <v>215</v>
       </c>
       <c r="B217" s="37" t="s">
-        <v>2177</v>
+        <v>2178</v>
       </c>
       <c r="C217" s="37">
         <v>1.0</v>
@@ -16688,7 +16688,7 @@
         <v>1328</v>
       </c>
       <c r="E217" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F217" s="39" t="s">
         <v>1691</v>
@@ -16697,10 +16697,10 @@
         <v>806</v>
       </c>
       <c r="H217" s="38" t="s">
-        <v>2178</v>
+        <v>2179</v>
       </c>
       <c r="I217" s="38" t="s">
-        <v>2178</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="218">
@@ -16718,7 +16718,7 @@
         <v>1330</v>
       </c>
       <c r="E218" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F218" s="39" t="s">
         <v>1691</v>
@@ -16727,10 +16727,10 @@
         <v>806</v>
       </c>
       <c r="H218" s="38" t="s">
-        <v>2179</v>
+        <v>2180</v>
       </c>
       <c r="I218" s="38" t="s">
-        <v>2179</v>
+        <v>2180</v>
       </c>
     </row>
     <row r="219">
@@ -16739,7 +16739,7 @@
         <v>217</v>
       </c>
       <c r="B219" s="37" t="s">
-        <v>2180</v>
+        <v>2181</v>
       </c>
       <c r="C219" s="37">
         <v>0.0</v>
@@ -16757,10 +16757,10 @@
         <v>806</v>
       </c>
       <c r="H219" s="38" t="s">
-        <v>2181</v>
+        <v>2182</v>
       </c>
       <c r="I219" s="38" t="s">
-        <v>2181</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="220">
@@ -16769,7 +16769,7 @@
         <v>218</v>
       </c>
       <c r="B220" s="37" t="s">
-        <v>2182</v>
+        <v>2183</v>
       </c>
       <c r="C220" s="37">
         <v>2.0</v>
@@ -16778,7 +16778,7 @@
         <v>1348</v>
       </c>
       <c r="E220" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F220" s="39" t="s">
         <v>806</v>
@@ -16787,10 +16787,10 @@
         <v>987</v>
       </c>
       <c r="H220" s="38" t="s">
-        <v>2183</v>
+        <v>2184</v>
       </c>
       <c r="I220" s="38" t="s">
-        <v>2184</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="221">
@@ -16799,7 +16799,7 @@
         <v>219</v>
       </c>
       <c r="B221" s="37" t="s">
-        <v>2185</v>
+        <v>2186</v>
       </c>
       <c r="C221" s="37">
         <v>1.0</v>
@@ -16808,7 +16808,7 @@
         <v>1334</v>
       </c>
       <c r="E221" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F221" s="39" t="s">
         <v>1691</v>
@@ -16817,10 +16817,10 @@
         <v>806</v>
       </c>
       <c r="H221" s="38" t="s">
-        <v>2186</v>
+        <v>2187</v>
       </c>
       <c r="I221" s="38" t="s">
-        <v>2186</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="222">
@@ -16829,7 +16829,7 @@
         <v>220</v>
       </c>
       <c r="B222" s="37" t="s">
-        <v>2187</v>
+        <v>2188</v>
       </c>
       <c r="C222" s="37">
         <v>0.0</v>
@@ -16847,10 +16847,10 @@
         <v>806</v>
       </c>
       <c r="H222" s="38" t="s">
-        <v>2188</v>
+        <v>2189</v>
       </c>
       <c r="I222" s="38" t="s">
-        <v>2188</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="223">
@@ -16859,7 +16859,7 @@
         <v>221</v>
       </c>
       <c r="B223" s="37" t="s">
-        <v>2189</v>
+        <v>2190</v>
       </c>
       <c r="C223" s="37">
         <v>1.0</v>
@@ -16868,7 +16868,7 @@
         <v>1338</v>
       </c>
       <c r="E223" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F223" s="39" t="s">
         <v>1691</v>
@@ -16877,10 +16877,10 @@
         <v>806</v>
       </c>
       <c r="H223" s="38" t="s">
-        <v>2190</v>
+        <v>2191</v>
       </c>
       <c r="I223" s="38" t="s">
-        <v>2190</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="224">
@@ -16889,7 +16889,7 @@
         <v>222</v>
       </c>
       <c r="B224" s="37" t="s">
-        <v>2191</v>
+        <v>2192</v>
       </c>
       <c r="C224" s="37">
         <v>0.0</v>
@@ -16907,10 +16907,10 @@
         <v>806</v>
       </c>
       <c r="H224" s="38" t="s">
-        <v>2192</v>
+        <v>2193</v>
       </c>
       <c r="I224" s="38" t="s">
-        <v>2192</v>
+        <v>2193</v>
       </c>
     </row>
     <row r="225">
@@ -16919,7 +16919,7 @@
         <v>223</v>
       </c>
       <c r="B225" s="37" t="s">
-        <v>2193</v>
+        <v>2194</v>
       </c>
       <c r="C225" s="37">
         <v>1.0</v>
@@ -16928,7 +16928,7 @@
         <v>1342</v>
       </c>
       <c r="E225" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F225" s="39" t="s">
         <v>1691</v>
@@ -16937,10 +16937,10 @@
         <v>806</v>
       </c>
       <c r="H225" s="38" t="s">
-        <v>2194</v>
+        <v>2195</v>
       </c>
       <c r="I225" s="38" t="s">
-        <v>2194</v>
+        <v>2195</v>
       </c>
     </row>
     <row r="226">
@@ -16967,10 +16967,10 @@
         <v>806</v>
       </c>
       <c r="H226" s="38" t="s">
-        <v>2195</v>
+        <v>2196</v>
       </c>
       <c r="I226" s="38" t="s">
-        <v>2195</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="227">
@@ -16979,7 +16979,7 @@
         <v>225</v>
       </c>
       <c r="B227" s="37" t="s">
-        <v>2196</v>
+        <v>2197</v>
       </c>
       <c r="C227" s="37">
         <v>1.0</v>
@@ -16988,7 +16988,7 @@
         <v>1344</v>
       </c>
       <c r="E227" s="39" t="s">
-        <v>964</v>
+        <v>2144</v>
       </c>
       <c r="F227" s="39" t="s">
         <v>1691</v>
@@ -16997,10 +16997,10 @@
         <v>806</v>
       </c>
       <c r="H227" s="38" t="s">
-        <v>2197</v>
+        <v>2198</v>
       </c>
       <c r="I227" s="38" t="s">
-        <v>2197</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="228">
@@ -17009,7 +17009,7 @@
         <v>226</v>
       </c>
       <c r="B228" s="37" t="s">
-        <v>2198</v>
+        <v>2199</v>
       </c>
       <c r="C228" s="37">
         <v>0.0</v>
@@ -17027,10 +17027,10 @@
         <v>806</v>
       </c>
       <c r="H228" s="38" t="s">
-        <v>2199</v>
+        <v>2200</v>
       </c>
       <c r="I228" s="38" t="s">
-        <v>2199</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="229">
@@ -17057,10 +17057,10 @@
         <v>806</v>
       </c>
       <c r="H229" s="38" t="s">
-        <v>2200</v>
+        <v>2201</v>
       </c>
       <c r="I229" s="38" t="s">
-        <v>2200</v>
+        <v>2201</v>
       </c>
     </row>
     <row r="230">
@@ -17087,10 +17087,10 @@
         <v>806</v>
       </c>
       <c r="H230" s="38" t="s">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="I230" s="38" t="s">
-        <v>2201</v>
+        <v>2202</v>
       </c>
     </row>
     <row r="231">
@@ -17099,7 +17099,7 @@
         <v>229</v>
       </c>
       <c r="B231" s="46" t="s">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="C231" s="65">
         <v>0.0</v>
@@ -17117,10 +17117,10 @@
         <v>806</v>
       </c>
       <c r="H231" s="42" t="s">
-        <v>2203</v>
+        <v>2204</v>
       </c>
       <c r="I231" s="42" t="s">
-        <v>2203</v>
+        <v>2204</v>
       </c>
     </row>
     <row r="232">
@@ -17129,7 +17129,7 @@
         <v>230</v>
       </c>
       <c r="B232" s="46" t="s">
-        <v>2204</v>
+        <v>2205</v>
       </c>
       <c r="C232" s="65">
         <v>1.0</v>
@@ -17137,8 +17137,8 @@
       <c r="D232" s="45" t="s">
         <v>1355</v>
       </c>
-      <c r="E232" s="53" t="s">
-        <v>964</v>
+      <c r="E232" s="39" t="s">
+        <v>2144</v>
       </c>
       <c r="F232" s="53" t="s">
         <v>1691</v>
@@ -17147,10 +17147,10 @@
         <v>806</v>
       </c>
       <c r="H232" s="42" t="s">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="I232" s="42" t="s">
-        <v>2205</v>
+        <v>2206</v>
       </c>
     </row>
     <row r="233">
@@ -17159,7 +17159,7 @@
         <v>231</v>
       </c>
       <c r="B233" s="46" t="s">
-        <v>2206</v>
+        <v>2207</v>
       </c>
       <c r="C233" s="46">
         <v>0.0</v>
@@ -17177,10 +17177,10 @@
         <v>806</v>
       </c>
       <c r="H233" s="42" t="s">
-        <v>2207</v>
+        <v>2208</v>
       </c>
       <c r="I233" s="42" t="s">
-        <v>2207</v>
+        <v>2208</v>
       </c>
     </row>
     <row r="234">
@@ -17189,7 +17189,7 @@
         <v>232</v>
       </c>
       <c r="B234" s="46" t="s">
-        <v>2208</v>
+        <v>2209</v>
       </c>
       <c r="C234" s="46">
         <v>1.0</v>
@@ -17197,8 +17197,8 @@
       <c r="D234" s="45" t="s">
         <v>1359</v>
       </c>
-      <c r="E234" s="45" t="s">
-        <v>964</v>
+      <c r="E234" s="39" t="s">
+        <v>2144</v>
       </c>
       <c r="F234" s="45" t="s">
         <v>1691</v>
@@ -17207,10 +17207,10 @@
         <v>806</v>
       </c>
       <c r="H234" s="42" t="s">
-        <v>2209</v>
+        <v>2210</v>
       </c>
       <c r="I234" s="42" t="s">
-        <v>2209</v>
+        <v>2210</v>
       </c>
     </row>
     <row r="235">
@@ -17219,7 +17219,7 @@
         <v>233</v>
       </c>
       <c r="B235" s="46" t="s">
-        <v>2210</v>
+        <v>2211</v>
       </c>
       <c r="C235" s="46">
         <v>0.0</v>
@@ -17237,10 +17237,10 @@
         <v>806</v>
       </c>
       <c r="H235" s="42" t="s">
-        <v>2211</v>
+        <v>2212</v>
       </c>
       <c r="I235" s="42" t="s">
-        <v>2211</v>
+        <v>2212</v>
       </c>
     </row>
     <row r="236">
@@ -17249,7 +17249,7 @@
         <v>234</v>
       </c>
       <c r="B236" s="46" t="s">
-        <v>2212</v>
+        <v>2213</v>
       </c>
       <c r="C236" s="46">
         <v>1.0</v>
@@ -17257,8 +17257,8 @@
       <c r="D236" s="45" t="s">
         <v>1363</v>
       </c>
-      <c r="E236" s="45" t="s">
-        <v>964</v>
+      <c r="E236" s="39" t="s">
+        <v>2144</v>
       </c>
       <c r="F236" s="45" t="s">
         <v>1691</v>
@@ -17267,10 +17267,10 @@
         <v>806</v>
       </c>
       <c r="H236" s="42" t="s">
-        <v>2213</v>
+        <v>2214</v>
       </c>
       <c r="I236" s="42" t="s">
-        <v>2213</v>
+        <v>2214</v>
       </c>
     </row>
     <row r="237">
@@ -17297,10 +17297,10 @@
         <v>806</v>
       </c>
       <c r="H237" s="42" t="s">
-        <v>2214</v>
+        <v>2215</v>
       </c>
       <c r="I237" s="42" t="s">
-        <v>2214</v>
+        <v>2215</v>
       </c>
     </row>
     <row r="238">
@@ -17309,7 +17309,7 @@
         <v>236</v>
       </c>
       <c r="B238" s="46" t="s">
-        <v>2215</v>
+        <v>2216</v>
       </c>
       <c r="C238" s="46">
         <v>0.0</v>
@@ -17327,10 +17327,10 @@
         <v>806</v>
       </c>
       <c r="H238" s="42" t="s">
-        <v>2216</v>
+        <v>2217</v>
       </c>
       <c r="I238" s="42" t="s">
-        <v>2216</v>
+        <v>2217</v>
       </c>
     </row>
     <row r="239">
@@ -17339,7 +17339,7 @@
         <v>237</v>
       </c>
       <c r="B239" s="46" t="s">
-        <v>2217</v>
+        <v>2218</v>
       </c>
       <c r="C239" s="46">
         <v>1.0</v>
@@ -17347,8 +17347,8 @@
       <c r="D239" s="45" t="s">
         <v>1369</v>
       </c>
-      <c r="E239" s="45" t="s">
-        <v>964</v>
+      <c r="E239" s="39" t="s">
+        <v>2144</v>
       </c>
       <c r="F239" s="45" t="s">
         <v>1691</v>
@@ -17357,10 +17357,10 @@
         <v>806</v>
       </c>
       <c r="H239" s="42" t="s">
-        <v>2218</v>
+        <v>2219</v>
       </c>
       <c r="I239" s="42" t="s">
-        <v>2218</v>
+        <v>2219</v>
       </c>
     </row>
     <row r="240">
@@ -17399,7 +17399,7 @@
         <v>239</v>
       </c>
       <c r="B241" s="37" t="s">
-        <v>2219</v>
+        <v>2220</v>
       </c>
       <c r="C241" s="37">
         <v>0.0</v>
@@ -17417,10 +17417,10 @@
         <v>806</v>
       </c>
       <c r="H241" s="38" t="s">
-        <v>2220</v>
+        <v>2221</v>
       </c>
       <c r="I241" s="38" t="s">
-        <v>2220</v>
+        <v>2221</v>
       </c>
     </row>
   </sheetData>
@@ -17462,34 +17462,34 @@
         <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2221</v>
+        <v>2222</v>
       </c>
       <c r="C1" s="29" t="s">
-        <v>2222</v>
+        <v>2223</v>
       </c>
       <c r="D1" s="29" t="s">
-        <v>2223</v>
+        <v>2224</v>
       </c>
       <c r="E1" s="29" t="s">
-        <v>2224</v>
+        <v>2225</v>
       </c>
       <c r="F1" s="29" t="s">
-        <v>2225</v>
+        <v>2226</v>
       </c>
       <c r="G1" s="29" t="s">
-        <v>2226</v>
+        <v>2227</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>2228</v>
+        <v>2229</v>
       </c>
       <c r="J1" s="66" t="s">
-        <v>2229</v>
+        <v>2230</v>
       </c>
       <c r="K1" s="66" t="s">
-        <v>2230</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="2" ht="186.0" customHeight="1">
@@ -17498,7 +17498,7 @@
         <v>-1</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>2231</v>
+        <v>2232</v>
       </c>
       <c r="C2" s="68" t="s">
         <v>337</v>
@@ -17534,7 +17534,7 @@
         <v>0</v>
       </c>
       <c r="B3" s="30" t="s">
-        <v>2232</v>
+        <v>2233</v>
       </c>
       <c r="C3" s="68" t="s">
         <v>1034</v>
@@ -17543,10 +17543,10 @@
         <v>1134</v>
       </c>
       <c r="E3" s="36" t="s">
-        <v>2233</v>
+        <v>2234</v>
       </c>
       <c r="F3" s="36" t="s">
-        <v>2234</v>
+        <v>2235</v>
       </c>
       <c r="G3" s="36" t="s">
         <v>335</v>
@@ -17570,19 +17570,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>2235</v>
+        <v>2236</v>
       </c>
       <c r="C4" s="68" t="s">
-        <v>2236</v>
+        <v>2237</v>
       </c>
       <c r="D4" s="69" t="s">
         <v>1134</v>
       </c>
       <c r="E4" s="36" t="s">
-        <v>2236</v>
+        <v>2237</v>
       </c>
       <c r="F4" s="36" t="s">
-        <v>2237</v>
+        <v>2238</v>
       </c>
       <c r="G4" s="36" t="s">
         <v>335</v>
@@ -17606,19 +17606,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>2238</v>
+        <v>2239</v>
       </c>
       <c r="C5" s="68" t="s">
-        <v>2239</v>
+        <v>2240</v>
       </c>
       <c r="D5" s="69" t="s">
         <v>1134</v>
       </c>
       <c r="E5" s="36" t="s">
-        <v>2239</v>
+        <v>2240</v>
       </c>
       <c r="F5" s="36" t="s">
-        <v>2240</v>
+        <v>2241</v>
       </c>
       <c r="G5" s="36" t="s">
         <v>335</v>
@@ -17642,19 +17642,19 @@
         <v>3</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>2241</v>
+        <v>2242</v>
       </c>
       <c r="C6" s="68" t="s">
-        <v>2242</v>
+        <v>2243</v>
       </c>
       <c r="D6" s="69" t="s">
         <v>1134</v>
       </c>
       <c r="E6" s="36" t="s">
-        <v>2242</v>
+        <v>2243</v>
       </c>
       <c r="F6" s="36" t="s">
-        <v>2243</v>
+        <v>2244</v>
       </c>
       <c r="G6" s="36" t="s">
         <v>335</v>
@@ -17678,25 +17678,25 @@
         <v>4</v>
       </c>
       <c r="B7" s="30" t="s">
-        <v>2244</v>
+        <v>2245</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>2245</v>
+        <v>2246</v>
       </c>
       <c r="D7" s="69" t="s">
+        <v>2247</v>
+      </c>
+      <c r="E7" s="36" t="s">
         <v>2246</v>
       </c>
-      <c r="E7" s="36" t="s">
-        <v>2245</v>
-      </c>
       <c r="F7" s="36" t="s">
-        <v>2247</v>
+        <v>2248</v>
       </c>
       <c r="G7" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H7" s="36" t="s">
-        <v>2246</v>
+        <v>2247</v>
       </c>
       <c r="I7" s="36" t="s">
         <v>705</v>
@@ -17714,25 +17714,25 @@
         <v>5</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>2248</v>
+        <v>2249</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>2249</v>
+        <v>2250</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>2246</v>
+        <v>2247</v>
       </c>
       <c r="E8" s="36" t="s">
-        <v>2249</v>
+        <v>2250</v>
       </c>
       <c r="F8" s="36" t="s">
-        <v>2250</v>
+        <v>2251</v>
       </c>
       <c r="G8" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H8" s="36" t="s">
-        <v>2246</v>
+        <v>2247</v>
       </c>
       <c r="I8" s="36" t="s">
         <v>705</v>
@@ -17750,7 +17750,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>2251</v>
+        <v>2252</v>
       </c>
       <c r="C9" s="33" t="s">
         <v>1071</v>
@@ -17762,7 +17762,7 @@
         <v>1071</v>
       </c>
       <c r="F9" s="36" t="s">
-        <v>2252</v>
+        <v>2253</v>
       </c>
       <c r="G9" s="36" t="s">
         <v>335</v>
@@ -17786,25 +17786,25 @@
         <v>7</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>2253</v>
+        <v>2254</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>2254</v>
+        <v>2255</v>
       </c>
       <c r="D10" s="69" t="s">
         <v>1130</v>
       </c>
       <c r="E10" s="36" t="s">
-        <v>2254</v>
+        <v>2255</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>2255</v>
+        <v>2256</v>
       </c>
       <c r="G10" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>2256</v>
+        <v>2257</v>
       </c>
       <c r="I10" s="36" t="s">
         <v>768</v>
@@ -17822,25 +17822,25 @@
         <v>8</v>
       </c>
       <c r="B11" s="30" t="s">
-        <v>2257</v>
+        <v>2258</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>2258</v>
+        <v>2259</v>
       </c>
       <c r="D11" s="69" t="s">
-        <v>2246</v>
+        <v>2247</v>
       </c>
       <c r="E11" s="36" t="s">
-        <v>2258</v>
+        <v>2259</v>
       </c>
       <c r="F11" s="36" t="s">
-        <v>2259</v>
+        <v>2260</v>
       </c>
       <c r="G11" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H11" s="36" t="s">
-        <v>2260</v>
+        <v>2261</v>
       </c>
       <c r="I11" s="36" t="s">
         <v>705</v>
@@ -17858,19 +17858,19 @@
         <v>9</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>2261</v>
+        <v>2262</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>2262</v>
+        <v>2263</v>
       </c>
       <c r="D12" s="69" t="s">
         <v>1129</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>2262</v>
+        <v>2263</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>2263</v>
+        <v>2264</v>
       </c>
       <c r="G12" s="36" t="s">
         <v>335</v>
@@ -17894,25 +17894,25 @@
         <v>10</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>2264</v>
+        <v>2265</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>2265</v>
+        <v>2266</v>
       </c>
       <c r="D13" s="69" t="s">
+        <v>2267</v>
+      </c>
+      <c r="E13" s="36" t="s">
         <v>2266</v>
       </c>
-      <c r="E13" s="36" t="s">
-        <v>2265</v>
-      </c>
       <c r="F13" s="36" t="s">
-        <v>2267</v>
+        <v>2268</v>
       </c>
       <c r="G13" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H13" s="36" t="s">
-        <v>2268</v>
+        <v>2269</v>
       </c>
       <c r="I13" s="36" t="s">
         <v>705</v>
@@ -17939,16 +17939,16 @@
         <v>21</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>2269</v>
+        <v>2270</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>2270</v>
+        <v>2271</v>
       </c>
       <c r="G14" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>2271</v>
+        <v>2272</v>
       </c>
       <c r="I14" s="36" t="s">
         <v>705</v>
@@ -17966,7 +17966,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>2272</v>
+        <v>2273</v>
       </c>
       <c r="C15" s="33" t="s">
         <v>1103</v>
@@ -17975,16 +17975,16 @@
         <v>21</v>
       </c>
       <c r="E15" s="36" t="s">
-        <v>2273</v>
+        <v>2274</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>2274</v>
+        <v>2275</v>
       </c>
       <c r="G15" s="36" t="s">
         <v>335</v>
       </c>
       <c r="H15" s="36" t="s">
-        <v>2275</v>
+        <v>2276</v>
       </c>
       <c r="I15" s="36" t="s">
         <v>705</v>
@@ -18002,7 +18002,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="30" t="s">
-        <v>2276</v>
+        <v>2277</v>
       </c>
       <c r="C16" s="68" t="s">
         <v>337</v>
@@ -18065,7 +18065,7 @@
         <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2277</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="2">
@@ -18092,7 +18092,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>2278</v>
+        <v>2279</v>
       </c>
     </row>
     <row r="5">
@@ -18101,7 +18101,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>2279</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="6">
@@ -18113,7 +18113,7 @@
         <v>50</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>2280</v>
+        <v>2281</v>
       </c>
     </row>
     <row r="8">
@@ -18121,7 +18121,7 @@
         <v>0.0</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>2281</v>
+        <v>2282</v>
       </c>
     </row>
     <row r="9">
@@ -18129,7 +18129,7 @@
         <v>1.0</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>2282</v>
+        <v>2283</v>
       </c>
     </row>
     <row r="10">
@@ -18137,7 +18137,7 @@
         <v>2.0</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>2283</v>
+        <v>2284</v>
       </c>
     </row>
     <row r="11">
@@ -18145,7 +18145,7 @@
         <v>3.0</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>2284</v>
+        <v>2285</v>
       </c>
     </row>
     <row r="12">
@@ -18153,7 +18153,7 @@
         <v>4.0</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>2285</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="13">
@@ -18161,7 +18161,7 @@
         <v>5.0</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>2286</v>
+        <v>2287</v>
       </c>
     </row>
     <row r="15">
@@ -18169,7 +18169,7 @@
         <v>50</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>2287</v>
+        <v>2288</v>
       </c>
     </row>
     <row r="16">
@@ -18187,7 +18187,7 @@
         <v>1</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>2288</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="18">
@@ -18232,7 +18232,7 @@
         <v>6</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>2289</v>
+        <v>2290</v>
       </c>
     </row>
     <row r="23">
@@ -18249,7 +18249,7 @@
         <v>50</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>2290</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="26">
@@ -18294,7 +18294,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>2291</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="31">
@@ -18348,7 +18348,7 @@
         <v>10</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>2292</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="37">
@@ -18428,10 +18428,10 @@
         <v>50</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>2293</v>
+        <v>2294</v>
       </c>
       <c r="C46" s="47" t="s">
-        <v>2294</v>
+        <v>2295</v>
       </c>
     </row>
     <row r="47">
@@ -18443,7 +18443,7 @@
         <v>806</v>
       </c>
       <c r="C47" s="37" t="s">
-        <v>2295</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="48">
@@ -18455,7 +18455,7 @@
         <v>1013</v>
       </c>
       <c r="C48" s="37" t="s">
-        <v>2296</v>
+        <v>2297</v>
       </c>
     </row>
     <row r="49">
@@ -18491,7 +18491,7 @@
         <v>5</v>
       </c>
       <c r="B52" s="37" t="s">
-        <v>2297</v>
+        <v>2298</v>
       </c>
     </row>
     <row r="53">
@@ -18500,7 +18500,7 @@
         <v>6</v>
       </c>
       <c r="B53" s="37" t="s">
-        <v>2298</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="54">
@@ -18509,7 +18509,7 @@
         <v>7</v>
       </c>
       <c r="B54" s="37" t="s">
-        <v>2299</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="55">
@@ -18518,7 +18518,7 @@
         <v>8</v>
       </c>
       <c r="B55" s="37" t="s">
-        <v>2300</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="56">
@@ -18527,7 +18527,7 @@
         <v>9</v>
       </c>
       <c r="B56" s="37" t="s">
-        <v>2301</v>
+        <v>2144</v>
       </c>
       <c r="C56" s="37" t="s">
         <v>2302</v>
@@ -20963,7 +20963,7 @@
         <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2280</v>
+        <v>2281</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
Unified Waypoint movement and order to al GameElements
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -722,13 +722,13 @@
     <t>If a Memento has been analyzed</t>
   </si>
   <si>
-    <t>INTERACT_PLAYER</t>
-  </si>
-  <si>
-    <t>INTERACT_PLAYER_DELEGATE</t>
-  </si>
-  <si>
-    <t>PlayerMasterClass.InteractPlayerService</t>
+    <t>INTERACT_ITEM</t>
+  </si>
+  <si>
+    <t>INTERACT_ITEM_DELEGATE</t>
+  </si>
+  <si>
+    <t>ItemMasterClass.InteractItemService</t>
   </si>
   <si>
     <t>Makes player interact with usage data</t>
@@ -746,13 +746,13 @@
     <t>Applies an unchain event to an item such as spawn or setsprite</t>
   </si>
   <si>
-    <t>PLAYER_REACHED_WAYPOINT</t>
-  </si>
-  <si>
-    <t>PLAYER_REACHED_WAYPOINT_DELEGATE</t>
-  </si>
-  <si>
-    <t>LevelMasterClass.PlayerReachedWaypointService</t>
+    <t>ITEM_REACHED_WAYPOINT</t>
+  </si>
+  <si>
+    <t>ITEM_REACHED_WAYPOINT_DELEGATE</t>
+  </si>
+  <si>
+    <t>LevelMasterClass.ItemReachedWaypointService</t>
   </si>
   <si>
     <t>Tells LevelMaster that player reached Waypoint to start action in case</t>
@@ -25965,10 +25965,10 @@
         <v>72</v>
       </c>
       <c r="N14" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="O14" s="13" t="s">
         <v>129</v>
-      </c>
-      <c r="O14" s="13" t="s">
-        <v>72</v>
       </c>
       <c r="P14" s="13" t="s">
         <v>72</v>
@@ -26421,10 +26421,10 @@
         <v>72</v>
       </c>
       <c r="N22" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="O22" s="24" t="s">
         <v>74</v>
-      </c>
-      <c r="O22" s="24" t="s">
-        <v>72</v>
       </c>
       <c r="P22" s="13" t="s">
         <v>72</v>
@@ -26545,10 +26545,10 @@
         <v>72</v>
       </c>
       <c r="N24" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="O24" s="24" t="s">
         <v>129</v>
-      </c>
-      <c r="O24" s="24" t="s">
-        <v>72</v>
       </c>
       <c r="P24" s="13" t="s">
         <v>72</v>
@@ -27590,7 +27590,7 @@
         <v>72</v>
       </c>
       <c r="I44" s="13" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="J44" s="13" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
Silvana walks. -Pending avoid a dead end if player saves just after using bladder -Pending auto resolve very small distances, as their assumed purpose is to flip X for different characters
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -45628,7 +45628,9 @@
       <c r="Q327" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="R327" s="38"/>
+      <c r="R327" s="38">
+        <v>0.0</v>
+      </c>
       <c r="S327" s="40" t="s">
         <v>874</v>
       </c>

</xml_diff>

<commit_message>
Encounter with alter Ego 1
</commit_message>
<xml_diff>
--- a/VARMAP_Generator/VARMAP.xlsx
+++ b/VARMAP_Generator/VARMAP.xlsx
@@ -7052,10 +7052,10 @@
     <t>NAME_DENIAL</t>
   </si>
   <si>
-    <t>Denial</t>
-  </si>
-  <si>
-    <t>Negación</t>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Hogar</t>
   </si>
   <si>
     <t>Portrait</t>
@@ -58692,7 +58692,7 @@
         <v>0.0</v>
       </c>
       <c r="V413" s="54">
-        <v>550.0</v>
+        <v>540.0</v>
       </c>
       <c r="W413" s="41" t="s">
         <v>948</v>
@@ -58902,7 +58902,7 @@
         <v>0.0</v>
       </c>
       <c r="V416" s="54">
-        <v>550.0</v>
+        <v>540.0</v>
       </c>
       <c r="W416" s="41" t="s">
         <v>948</v>

</xml_diff>